<commit_message>
feat: ship on-site updates and keyboard-safe Modern dialogs
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="Re490b7bd213a4afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R03036dd6d17d462c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF416B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2B8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -190,7 +200,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="95">
+  <x:cellXfs count="110">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -472,6 +482,51 @@
     <x:xf numFmtId="0" fontId="4" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -480,8 +535,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2818" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H2818"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2829" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H2829"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Раздел"/>
     <x:tableColumn id="2" name="ID (не менять)"/>
@@ -67503,10 +67558,230 @@
       <x:c r="G2818" s="93" t="str"/>
       <x:c r="H2818" s="94" t="str"/>
     </x:row>
+    <x:row r="2819" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2819" s="101" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2819" s="101" t="str">
+        <x:v>shell.skipCalculator</x:v>
+      </x:c>
+      <x:c r="C2819" s="101" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2819" s="102" t="str"/>
+      <x:c r="E2819" s="102" t="str">
+        <x:v>Skip to calculator</x:v>
+      </x:c>
+      <x:c r="F2819" s="102" t="str"/>
+      <x:c r="G2819" s="102" t="str"/>
+      <x:c r="H2819" s="103" t="str">
+        <x:v>Перейти к калькулятору</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2820" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2820" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2820" s="104" t="str">
+        <x:v>updates.title</x:v>
+      </x:c>
+      <x:c r="C2820" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2820" s="105" t="str"/>
+      <x:c r="E2820" s="105" t="str">
+        <x:v>What's new</x:v>
+      </x:c>
+      <x:c r="F2820" s="105" t="str"/>
+      <x:c r="G2820" s="105" t="str"/>
+      <x:c r="H2820" s="106" t="str">
+        <x:v>Что нового</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2821" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2821" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2821" s="104" t="str">
+        <x:v>updates.close</x:v>
+      </x:c>
+      <x:c r="C2821" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2821" s="105" t="str"/>
+      <x:c r="E2821" s="105" t="str">
+        <x:v>Close updates</x:v>
+      </x:c>
+      <x:c r="F2821" s="105" t="str"/>
+      <x:c r="G2821" s="105" t="str"/>
+      <x:c r="H2821" s="106" t="str">
+        <x:v>Закрыть обновления</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2822" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2822" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2822" s="104" t="str">
+        <x:v>updates.version</x:v>
+      </x:c>
+      <x:c r="C2822" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2822" s="105" t="str"/>
+      <x:c r="E2822" s="105" t="str">
+        <x:v>Legacy engine: {legacyEngine} · Remaked UI: {ui}</x:v>
+      </x:c>
+      <x:c r="F2822" s="105" t="str"/>
+      <x:c r="G2822" s="105" t="str"/>
+      <x:c r="H2822" s="106" t="str">
+        <x:v>Legacy engine: {legacyEngine} · Remaked UI: {ui}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2823" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2823" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2823" s="104" t="str">
+        <x:v>updates.keyboard</x:v>
+      </x:c>
+      <x:c r="C2823" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2823" s="105" t="str"/>
+      <x:c r="E2823" s="105" t="str">
+        <x:v>Keyboard navigation: skip straight to the calculator, keep focus inside open dialogs, and return to the opener with Escape.</x:v>
+      </x:c>
+      <x:c r="F2823" s="105" t="str"/>
+      <x:c r="G2823" s="105" t="str"/>
+      <x:c r="H2823" s="106" t="str">
+        <x:v>Управление клавиатурой: переходите сразу к калькулятору, оставайтесь внутри открытого окна и возвращайтесь к кнопке открытия через Escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2824" ht="48" hidden="0" customHeight="1">
+      <x:c r="A2824" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2824" s="104" t="str">
+        <x:v>updates.translations</x:v>
+      </x:c>
+      <x:c r="C2824" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2824" s="105" t="str"/>
+      <x:c r="E2824" s="105" t="str">
+        <x:v>Translate the Modern interface, game names, labels and skill descriptions in one Excel workbook. Upload it to GitHub to publish an update.</x:v>
+      </x:c>
+      <x:c r="F2824" s="105" t="str"/>
+      <x:c r="G2824" s="105" t="str"/>
+      <x:c r="H2824" s="106" t="str">
+        <x:v>Переводите современный интерфейс, игровые названия, подписи и описания навыков в одной Excel-таблице. Загрузите её на GitHub, чтобы опубликовать обновление.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2825" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2825" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2825" s="104" t="str">
+        <x:v>updates.builds</x:v>
+      </x:c>
+      <x:c r="C2825" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2825" s="105" t="str"/>
+      <x:c r="E2825" s="105" t="str">
+        <x:v>Search compatible equipment and Souls, save named builds locally, and compare their calculated stats without changing your current character.</x:v>
+      </x:c>
+      <x:c r="F2825" s="105" t="str"/>
+      <x:c r="G2825" s="105" t="str"/>
+      <x:c r="H2825" s="106" t="str">
+        <x:v>Ищите подходящую экипировку и Souls, сохраняйте билды в браузере и сравнивайте рассчитанные характеристики без изменения текущего персонажа.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2826" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2826" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2826" s="104" t="str">
+        <x:v>updates.offline</x:v>
+      </x:c>
+      <x:c r="C2826" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2826" s="105" t="str"/>
+      <x:c r="E2826" s="105" t="str">
+        <x:v>Install the site or use Modern and Legacy modes offline after the first successful load. Save your work before accepting an update.</x:v>
+      </x:c>
+      <x:c r="F2826" s="105" t="str"/>
+      <x:c r="G2826" s="105" t="str"/>
+      <x:c r="H2826" s="106" t="str">
+        <x:v>Установите сайт или используйте Modern и Legacy офлайн после первой успешной загрузки. Сохраните работу перед обновлением.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2827" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2827" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2827" s="104" t="str">
+        <x:v>updates.preservation</x:v>
+      </x:c>
+      <x:c r="C2827" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2827" s="105" t="str"/>
+      <x:c r="E2827" s="105" t="str">
+        <x:v>The Legacy 2.00 engine remains the calculation source. This is an unofficial community project. Build storage is local to this browser.</x:v>
+      </x:c>
+      <x:c r="F2827" s="105" t="str"/>
+      <x:c r="G2827" s="105" t="str"/>
+      <x:c r="H2827" s="106" t="str">
+        <x:v>Источником расчётов остаётся движок Legacy 2.00. Это неофициальный проект сообщества. Билды хранятся только в этом браузере.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2828" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2828" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2828" s="104" t="str">
+        <x:v>updates.fullChangelog</x:v>
+      </x:c>
+      <x:c r="C2828" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2828" s="105" t="str"/>
+      <x:c r="E2828" s="105" t="str">
+        <x:v>Full changelog</x:v>
+      </x:c>
+      <x:c r="F2828" s="105" t="str"/>
+      <x:c r="G2828" s="105" t="str"/>
+      <x:c r="H2828" s="106" t="str">
+        <x:v>Полный список изменений</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2829" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2829" s="107" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2829" s="107" t="str">
+        <x:v>updates.report</x:v>
+      </x:c>
+      <x:c r="C2829" s="107" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2829" s="108" t="str"/>
+      <x:c r="E2829" s="108" t="str">
+        <x:v>Report a problem</x:v>
+      </x:c>
+      <x:c r="F2829" s="108" t="str"/>
+      <x:c r="G2829" s="108" t="str"/>
+      <x:c r="H2829" s="109" t="str">
+        <x:v>Сообщить о проблеме</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d2948c84ff34ebe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf227ad6dce8741f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
On-site updates and keyboard-safe Modern dialogs (#14)
* test: start Phase 7 cross-browser acceptance gates

* feat: ship on-site updates and keyboard-safe Modern dialogs
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="Re490b7bd213a4afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R03036dd6d17d462c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF416B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2B8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -190,7 +200,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="95">
+  <x:cellXfs count="110">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -472,6 +482,51 @@
     <x:xf numFmtId="0" fontId="4" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -480,8 +535,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2818" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H2818"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2829" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H2829"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Раздел"/>
     <x:tableColumn id="2" name="ID (не менять)"/>
@@ -67503,10 +67558,230 @@
       <x:c r="G2818" s="93" t="str"/>
       <x:c r="H2818" s="94" t="str"/>
     </x:row>
+    <x:row r="2819" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2819" s="101" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2819" s="101" t="str">
+        <x:v>shell.skipCalculator</x:v>
+      </x:c>
+      <x:c r="C2819" s="101" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2819" s="102" t="str"/>
+      <x:c r="E2819" s="102" t="str">
+        <x:v>Skip to calculator</x:v>
+      </x:c>
+      <x:c r="F2819" s="102" t="str"/>
+      <x:c r="G2819" s="102" t="str"/>
+      <x:c r="H2819" s="103" t="str">
+        <x:v>Перейти к калькулятору</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2820" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2820" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2820" s="104" t="str">
+        <x:v>updates.title</x:v>
+      </x:c>
+      <x:c r="C2820" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2820" s="105" t="str"/>
+      <x:c r="E2820" s="105" t="str">
+        <x:v>What's new</x:v>
+      </x:c>
+      <x:c r="F2820" s="105" t="str"/>
+      <x:c r="G2820" s="105" t="str"/>
+      <x:c r="H2820" s="106" t="str">
+        <x:v>Что нового</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2821" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2821" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2821" s="104" t="str">
+        <x:v>updates.close</x:v>
+      </x:c>
+      <x:c r="C2821" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2821" s="105" t="str"/>
+      <x:c r="E2821" s="105" t="str">
+        <x:v>Close updates</x:v>
+      </x:c>
+      <x:c r="F2821" s="105" t="str"/>
+      <x:c r="G2821" s="105" t="str"/>
+      <x:c r="H2821" s="106" t="str">
+        <x:v>Закрыть обновления</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2822" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2822" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2822" s="104" t="str">
+        <x:v>updates.version</x:v>
+      </x:c>
+      <x:c r="C2822" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2822" s="105" t="str"/>
+      <x:c r="E2822" s="105" t="str">
+        <x:v>Legacy engine: {legacyEngine} · Remaked UI: {ui}</x:v>
+      </x:c>
+      <x:c r="F2822" s="105" t="str"/>
+      <x:c r="G2822" s="105" t="str"/>
+      <x:c r="H2822" s="106" t="str">
+        <x:v>Legacy engine: {legacyEngine} · Remaked UI: {ui}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2823" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2823" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2823" s="104" t="str">
+        <x:v>updates.keyboard</x:v>
+      </x:c>
+      <x:c r="C2823" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2823" s="105" t="str"/>
+      <x:c r="E2823" s="105" t="str">
+        <x:v>Keyboard navigation: skip straight to the calculator, keep focus inside open dialogs, and return to the opener with Escape.</x:v>
+      </x:c>
+      <x:c r="F2823" s="105" t="str"/>
+      <x:c r="G2823" s="105" t="str"/>
+      <x:c r="H2823" s="106" t="str">
+        <x:v>Управление клавиатурой: переходите сразу к калькулятору, оставайтесь внутри открытого окна и возвращайтесь к кнопке открытия через Escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2824" ht="48" hidden="0" customHeight="1">
+      <x:c r="A2824" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2824" s="104" t="str">
+        <x:v>updates.translations</x:v>
+      </x:c>
+      <x:c r="C2824" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2824" s="105" t="str"/>
+      <x:c r="E2824" s="105" t="str">
+        <x:v>Translate the Modern interface, game names, labels and skill descriptions in one Excel workbook. Upload it to GitHub to publish an update.</x:v>
+      </x:c>
+      <x:c r="F2824" s="105" t="str"/>
+      <x:c r="G2824" s="105" t="str"/>
+      <x:c r="H2824" s="106" t="str">
+        <x:v>Переводите современный интерфейс, игровые названия, подписи и описания навыков в одной Excel-таблице. Загрузите её на GitHub, чтобы опубликовать обновление.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2825" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2825" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2825" s="104" t="str">
+        <x:v>updates.builds</x:v>
+      </x:c>
+      <x:c r="C2825" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2825" s="105" t="str"/>
+      <x:c r="E2825" s="105" t="str">
+        <x:v>Search compatible equipment and Souls, save named builds locally, and compare their calculated stats without changing your current character.</x:v>
+      </x:c>
+      <x:c r="F2825" s="105" t="str"/>
+      <x:c r="G2825" s="105" t="str"/>
+      <x:c r="H2825" s="106" t="str">
+        <x:v>Ищите подходящую экипировку и Souls, сохраняйте билды в браузере и сравнивайте рассчитанные характеристики без изменения текущего персонажа.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2826" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2826" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2826" s="104" t="str">
+        <x:v>updates.offline</x:v>
+      </x:c>
+      <x:c r="C2826" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2826" s="105" t="str"/>
+      <x:c r="E2826" s="105" t="str">
+        <x:v>Install the site or use Modern and Legacy modes offline after the first successful load. Save your work before accepting an update.</x:v>
+      </x:c>
+      <x:c r="F2826" s="105" t="str"/>
+      <x:c r="G2826" s="105" t="str"/>
+      <x:c r="H2826" s="106" t="str">
+        <x:v>Установите сайт или используйте Modern и Legacy офлайн после первой успешной загрузки. Сохраните работу перед обновлением.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2827" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2827" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2827" s="104" t="str">
+        <x:v>updates.preservation</x:v>
+      </x:c>
+      <x:c r="C2827" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2827" s="105" t="str"/>
+      <x:c r="E2827" s="105" t="str">
+        <x:v>The Legacy 2.00 engine remains the calculation source. This is an unofficial community project. Build storage is local to this browser.</x:v>
+      </x:c>
+      <x:c r="F2827" s="105" t="str"/>
+      <x:c r="G2827" s="105" t="str"/>
+      <x:c r="H2827" s="106" t="str">
+        <x:v>Источником расчётов остаётся движок Legacy 2.00. Это неофициальный проект сообщества. Билды хранятся только в этом браузере.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2828" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2828" s="104" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2828" s="104" t="str">
+        <x:v>updates.fullChangelog</x:v>
+      </x:c>
+      <x:c r="C2828" s="104" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2828" s="105" t="str"/>
+      <x:c r="E2828" s="105" t="str">
+        <x:v>Full changelog</x:v>
+      </x:c>
+      <x:c r="F2828" s="105" t="str"/>
+      <x:c r="G2828" s="105" t="str"/>
+      <x:c r="H2828" s="106" t="str">
+        <x:v>Полный список изменений</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2829" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2829" s="107" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2829" s="107" t="str">
+        <x:v>updates.report</x:v>
+      </x:c>
+      <x:c r="C2829" s="107" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2829" s="108" t="str"/>
+      <x:c r="E2829" s="108" t="str">
+        <x:v>Report a problem</x:v>
+      </x:c>
+      <x:c r="F2829" s="108" t="str"/>
+      <x:c r="G2829" s="108" t="str"/>
+      <x:c r="H2829" s="109" t="str">
+        <x:v>Сообщить о проблеме</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d2948c84ff34ebe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf227ad6dce8741f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Unify Modern UI, item previews and reliable build sharing
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R03036dd6d17d462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R2dca05788e9d4091"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF416B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2B8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -200,7 +210,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="110">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -527,6 +537,51 @@
     <x:xf numFmtId="0" fontId="4" fillId="16" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -535,8 +590,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2829" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H2829"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2838" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H2838"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Раздел"/>
     <x:tableColumn id="2" name="ID (не менять)"/>
@@ -67778,10 +67833,190 @@
         <x:v>Сообщить о проблеме</x:v>
       </x:c>
     </x:row>
+    <x:row r="2830" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2830" s="116" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2830" s="116" t="str">
+        <x:v>builds.share</x:v>
+      </x:c>
+      <x:c r="C2830" s="116" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2830" s="117" t="str"/>
+      <x:c r="E2830" s="117" t="str">
+        <x:v>Share build</x:v>
+      </x:c>
+      <x:c r="F2830" s="117" t="str"/>
+      <x:c r="G2830" s="117" t="str"/>
+      <x:c r="H2830" s="118" t="str">
+        <x:v>Поделиться билдом</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2831" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2831" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2831" s="119" t="str">
+        <x:v>builds.shareLink</x:v>
+      </x:c>
+      <x:c r="C2831" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2831" s="120" t="str"/>
+      <x:c r="E2831" s="120" t="str">
+        <x:v>Build sharing link</x:v>
+      </x:c>
+      <x:c r="F2831" s="120" t="str"/>
+      <x:c r="G2831" s="120" t="str"/>
+      <x:c r="H2831" s="121" t="str">
+        <x:v>Ссылка на билд</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2832" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2832" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2832" s="119" t="str">
+        <x:v>builds.shareCopied</x:v>
+      </x:c>
+      <x:c r="C2832" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2832" s="120" t="str"/>
+      <x:c r="E2832" s="120" t="str">
+        <x:v>Build link copied.</x:v>
+      </x:c>
+      <x:c r="F2832" s="120" t="str"/>
+      <x:c r="G2832" s="120" t="str"/>
+      <x:c r="H2832" s="121" t="str">
+        <x:v>Ссылка на билд скопирована.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2833" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2833" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2833" s="119" t="str">
+        <x:v>builds.shareManual</x:v>
+      </x:c>
+      <x:c r="C2833" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2833" s="120" t="str"/>
+      <x:c r="E2833" s="120" t="str">
+        <x:v>Copy the link below to share your build.</x:v>
+      </x:c>
+      <x:c r="F2833" s="120" t="str"/>
+      <x:c r="G2833" s="120" t="str"/>
+      <x:c r="H2833" s="121" t="str">
+        <x:v>Скопируйте ссылку ниже, чтобы поделиться билдом.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2834" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2834" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2834" s="119" t="str">
+        <x:v>builds.sharedLoaded</x:v>
+      </x:c>
+      <x:c r="C2834" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2834" s="120" t="str"/>
+      <x:c r="E2834" s="120" t="str">
+        <x:v>Shared build loaded</x:v>
+      </x:c>
+      <x:c r="F2834" s="120" t="str"/>
+      <x:c r="G2834" s="120" t="str"/>
+      <x:c r="H2834" s="121" t="str">
+        <x:v>Билд из ссылки загружен</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2835" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2835" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2835" s="119" t="str">
+        <x:v>builds.invalidShare</x:v>
+      </x:c>
+      <x:c r="C2835" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2835" s="120" t="str"/>
+      <x:c r="E2835" s="120" t="str">
+        <x:v>Invalid share link; current build kept</x:v>
+      </x:c>
+      <x:c r="F2835" s="120" t="str"/>
+      <x:c r="G2835" s="120" t="str"/>
+      <x:c r="H2835" s="121" t="str">
+        <x:v>Некорректная ссылка; текущий билд сохранён</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2836" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2836" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2836" s="119" t="str">
+        <x:v>search.details</x:v>
+      </x:c>
+      <x:c r="C2836" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2836" s="120" t="str"/>
+      <x:c r="E2836" s="120" t="str">
+        <x:v>Details</x:v>
+      </x:c>
+      <x:c r="F2836" s="120" t="str"/>
+      <x:c r="G2836" s="120" t="str"/>
+      <x:c r="H2836" s="121" t="str">
+        <x:v>Характеристики</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2837" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2837" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2837" s="119" t="str">
+        <x:v>search.sockets</x:v>
+      </x:c>
+      <x:c r="C2837" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2837" s="120" t="str"/>
+      <x:c r="E2837" s="120" t="str">
+        <x:v>Soul sockets: {count}</x:v>
+      </x:c>
+      <x:c r="F2837" s="120" t="str"/>
+      <x:c r="G2837" s="120" t="str"/>
+      <x:c r="H2837" s="121" t="str">
+        <x:v>Ячеек Soul: {count}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2838" ht="24" hidden="0" customHeight="1">
+      <x:c r="A2838" s="122" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2838" s="122" t="str">
+        <x:v>search.itemSource</x:v>
+      </x:c>
+      <x:c r="C2838" s="122" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2838" s="123" t="str"/>
+      <x:c r="E2838" s="123" t="str">
+        <x:v>Item descriptions from Legacy 2.00; not calculated build deltas.</x:v>
+      </x:c>
+      <x:c r="F2838" s="123" t="str"/>
+      <x:c r="G2838" s="123" t="str"/>
+      <x:c r="H2838" s="124" t="str">
+        <x:v>Описание предмета из Legacy 2.00; это не расчёт изменений характеристик билда.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf227ad6dce8741f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2307a5e74eb4215"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Unify Modern UI, item previews and reliable build sharing (#16)
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R03036dd6d17d462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R2dca05788e9d4091"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF416B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2B8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -200,7 +210,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="110">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -527,6 +537,51 @@
     <x:xf numFmtId="0" fontId="4" fillId="16" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="18" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -535,8 +590,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2829" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H2829"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2838" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H2838"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Раздел"/>
     <x:tableColumn id="2" name="ID (не менять)"/>
@@ -67778,10 +67833,190 @@
         <x:v>Сообщить о проблеме</x:v>
       </x:c>
     </x:row>
+    <x:row r="2830" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2830" s="116" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2830" s="116" t="str">
+        <x:v>builds.share</x:v>
+      </x:c>
+      <x:c r="C2830" s="116" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2830" s="117" t="str"/>
+      <x:c r="E2830" s="117" t="str">
+        <x:v>Share build</x:v>
+      </x:c>
+      <x:c r="F2830" s="117" t="str"/>
+      <x:c r="G2830" s="117" t="str"/>
+      <x:c r="H2830" s="118" t="str">
+        <x:v>Поделиться билдом</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2831" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2831" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2831" s="119" t="str">
+        <x:v>builds.shareLink</x:v>
+      </x:c>
+      <x:c r="C2831" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2831" s="120" t="str"/>
+      <x:c r="E2831" s="120" t="str">
+        <x:v>Build sharing link</x:v>
+      </x:c>
+      <x:c r="F2831" s="120" t="str"/>
+      <x:c r="G2831" s="120" t="str"/>
+      <x:c r="H2831" s="121" t="str">
+        <x:v>Ссылка на билд</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2832" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2832" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2832" s="119" t="str">
+        <x:v>builds.shareCopied</x:v>
+      </x:c>
+      <x:c r="C2832" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2832" s="120" t="str"/>
+      <x:c r="E2832" s="120" t="str">
+        <x:v>Build link copied.</x:v>
+      </x:c>
+      <x:c r="F2832" s="120" t="str"/>
+      <x:c r="G2832" s="120" t="str"/>
+      <x:c r="H2832" s="121" t="str">
+        <x:v>Ссылка на билд скопирована.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2833" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2833" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2833" s="119" t="str">
+        <x:v>builds.shareManual</x:v>
+      </x:c>
+      <x:c r="C2833" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2833" s="120" t="str"/>
+      <x:c r="E2833" s="120" t="str">
+        <x:v>Copy the link below to share your build.</x:v>
+      </x:c>
+      <x:c r="F2833" s="120" t="str"/>
+      <x:c r="G2833" s="120" t="str"/>
+      <x:c r="H2833" s="121" t="str">
+        <x:v>Скопируйте ссылку ниже, чтобы поделиться билдом.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2834" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2834" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2834" s="119" t="str">
+        <x:v>builds.sharedLoaded</x:v>
+      </x:c>
+      <x:c r="C2834" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2834" s="120" t="str"/>
+      <x:c r="E2834" s="120" t="str">
+        <x:v>Shared build loaded</x:v>
+      </x:c>
+      <x:c r="F2834" s="120" t="str"/>
+      <x:c r="G2834" s="120" t="str"/>
+      <x:c r="H2834" s="121" t="str">
+        <x:v>Билд из ссылки загружен</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2835" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2835" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2835" s="119" t="str">
+        <x:v>builds.invalidShare</x:v>
+      </x:c>
+      <x:c r="C2835" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2835" s="120" t="str"/>
+      <x:c r="E2835" s="120" t="str">
+        <x:v>Invalid share link; current build kept</x:v>
+      </x:c>
+      <x:c r="F2835" s="120" t="str"/>
+      <x:c r="G2835" s="120" t="str"/>
+      <x:c r="H2835" s="121" t="str">
+        <x:v>Некорректная ссылка; текущий билд сохранён</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2836" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2836" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2836" s="119" t="str">
+        <x:v>search.details</x:v>
+      </x:c>
+      <x:c r="C2836" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2836" s="120" t="str"/>
+      <x:c r="E2836" s="120" t="str">
+        <x:v>Details</x:v>
+      </x:c>
+      <x:c r="F2836" s="120" t="str"/>
+      <x:c r="G2836" s="120" t="str"/>
+      <x:c r="H2836" s="121" t="str">
+        <x:v>Характеристики</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2837" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2837" s="119" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2837" s="119" t="str">
+        <x:v>search.sockets</x:v>
+      </x:c>
+      <x:c r="C2837" s="119" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2837" s="120" t="str"/>
+      <x:c r="E2837" s="120" t="str">
+        <x:v>Soul sockets: {count}</x:v>
+      </x:c>
+      <x:c r="F2837" s="120" t="str"/>
+      <x:c r="G2837" s="120" t="str"/>
+      <x:c r="H2837" s="121" t="str">
+        <x:v>Ячеек Soul: {count}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2838" ht="24" hidden="0" customHeight="1">
+      <x:c r="A2838" s="122" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2838" s="122" t="str">
+        <x:v>search.itemSource</x:v>
+      </x:c>
+      <x:c r="C2838" s="122" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2838" s="123" t="str"/>
+      <x:c r="E2838" s="123" t="str">
+        <x:v>Item descriptions from Legacy 2.00; not calculated build deltas.</x:v>
+      </x:c>
+      <x:c r="F2838" s="123" t="str"/>
+      <x:c r="G2838" s="123" t="str"/>
+      <x:c r="H2838" s="124" t="str">
+        <x:v>Описание предмета из Legacy 2.00; это не расчёт изменений характеристик билда.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf227ad6dce8741f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2307a5e74eb4215"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve skill allocation and explicit effect controls
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R2dca05788e9d4091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R04e8a8caf1d84324"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF416B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2B8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -210,7 +220,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="125">
+  <x:cellXfs count="140">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -582,6 +592,51 @@
     <x:xf numFmtId="0" fontId="4" fillId="18" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -590,8 +645,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2838" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H2838"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2843" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H2843"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Раздел"/>
     <x:tableColumn id="2" name="ID (не менять)"/>
@@ -68013,10 +68068,104 @@
         <x:v>Описание предмета из Legacy 2.00; это не расчёт изменений характеристик билда.</x:v>
       </x:c>
     </x:row>
+    <x:row r="2839" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2839" s="131" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2839" s="131" t="str">
+        <x:v>skills.adeptness</x:v>
+      </x:c>
+      <x:c r="C2839" s="131" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2839" s="132" t="str"/>
+      <x:c r="E2839" s="132" t="str">
+        <x:v>Adeptness</x:v>
+      </x:c>
+      <x:c r="F2839" s="132" t="str"/>
+      <x:c r="G2839" s="132" t="str"/>
+      <x:c r="H2839" s="133" t="str"/>
+    </x:row>
+    <x:row r="2840" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2840" s="134" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2840" s="134" t="str">
+        <x:v>skills.potential</x:v>
+      </x:c>
+      <x:c r="C2840" s="134" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2840" s="135" t="str"/>
+      <x:c r="E2840" s="135" t="str">
+        <x:v>Potential</x:v>
+      </x:c>
+      <x:c r="F2840" s="135" t="str"/>
+      <x:c r="G2840" s="135" t="str"/>
+      <x:c r="H2840" s="136" t="str"/>
+    </x:row>
+    <x:row r="2841" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2841" s="134" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2841" s="134" t="str">
+        <x:v>skills.largerSteps</x:v>
+      </x:c>
+      <x:c r="C2841" s="134" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2841" s="135" t="str"/>
+      <x:c r="E2841" s="135" t="str">
+        <x:v>Larger steps</x:v>
+      </x:c>
+      <x:c r="F2841" s="135" t="str"/>
+      <x:c r="G2841" s="135" t="str"/>
+      <x:c r="H2841" s="136" t="str">
+        <x:v>Крупные шаги</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2842" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2842" s="134" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2842" s="134" t="str">
+        <x:v>skills.help</x:v>
+      </x:c>
+      <x:c r="C2842" s="134" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2842" s="135" t="str"/>
+      <x:c r="E2842" s="135" t="str">
+        <x:v>Adeptness uses Skill points. Potential uses its own point pool beside Level. Limits and costs follow the Legacy engine.</x:v>
+      </x:c>
+      <x:c r="F2842" s="135" t="str"/>
+      <x:c r="G2842" s="135" t="str"/>
+      <x:c r="H2842" s="136" t="str">
+        <x:v>Adeptness использует очки Skill. Potential использует свой запас очков рядом с уровнем. Ограничения и стоимость определяет движок Legacy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2843" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2843" s="137" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2843" s="137" t="str">
+        <x:v>skills.indicator</x:v>
+      </x:c>
+      <x:c r="C2843" s="137" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2843" s="138" t="str"/>
+      <x:c r="E2843" s="138" t="str">
+        <x:v>Legacy next-point indicator: </x:v>
+      </x:c>
+      <x:c r="F2843" s="138" t="str"/>
+      <x:c r="G2843" s="138" t="str"/>
+      <x:c r="H2843" s="139" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2307a5e74eb4215"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c0af64477a4a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve skill allocation and explicit effect controls (#22)
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R2dca05788e9d4091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переводы" sheetId="1" r:id="R04e8a8caf1d84324"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF416B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2B8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -210,7 +220,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="125">
+  <x:cellXfs count="140">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -582,6 +592,51 @@
     <x:xf numFmtId="0" fontId="4" fillId="18" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -590,8 +645,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2838" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H2838"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:H2843" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H2843"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Раздел"/>
     <x:tableColumn id="2" name="ID (не менять)"/>
@@ -68013,10 +68068,104 @@
         <x:v>Описание предмета из Legacy 2.00; это не расчёт изменений характеристик билда.</x:v>
       </x:c>
     </x:row>
+    <x:row r="2839" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2839" s="131" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2839" s="131" t="str">
+        <x:v>skills.adeptness</x:v>
+      </x:c>
+      <x:c r="C2839" s="131" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2839" s="132" t="str"/>
+      <x:c r="E2839" s="132" t="str">
+        <x:v>Adeptness</x:v>
+      </x:c>
+      <x:c r="F2839" s="132" t="str"/>
+      <x:c r="G2839" s="132" t="str"/>
+      <x:c r="H2839" s="133" t="str"/>
+    </x:row>
+    <x:row r="2840" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2840" s="134" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2840" s="134" t="str">
+        <x:v>skills.potential</x:v>
+      </x:c>
+      <x:c r="C2840" s="134" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2840" s="135" t="str"/>
+      <x:c r="E2840" s="135" t="str">
+        <x:v>Potential</x:v>
+      </x:c>
+      <x:c r="F2840" s="135" t="str"/>
+      <x:c r="G2840" s="135" t="str"/>
+      <x:c r="H2840" s="136" t="str"/>
+    </x:row>
+    <x:row r="2841" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2841" s="134" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2841" s="134" t="str">
+        <x:v>skills.largerSteps</x:v>
+      </x:c>
+      <x:c r="C2841" s="134" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2841" s="135" t="str"/>
+      <x:c r="E2841" s="135" t="str">
+        <x:v>Larger steps</x:v>
+      </x:c>
+      <x:c r="F2841" s="135" t="str"/>
+      <x:c r="G2841" s="135" t="str"/>
+      <x:c r="H2841" s="136" t="str">
+        <x:v>Крупные шаги</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2842" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2842" s="134" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2842" s="134" t="str">
+        <x:v>skills.help</x:v>
+      </x:c>
+      <x:c r="C2842" s="134" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2842" s="135" t="str"/>
+      <x:c r="E2842" s="135" t="str">
+        <x:v>Adeptness uses Skill points. Potential uses its own point pool beside Level. Limits and costs follow the Legacy engine.</x:v>
+      </x:c>
+      <x:c r="F2842" s="135" t="str"/>
+      <x:c r="G2842" s="135" t="str"/>
+      <x:c r="H2842" s="136" t="str">
+        <x:v>Adeptness использует очки Skill. Potential использует свой запас очков рядом с уровнем. Ограничения и стоимость определяет движок Legacy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2843" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2843" s="137" t="str">
+        <x:v>Интерфейс</x:v>
+      </x:c>
+      <x:c r="B2843" s="137" t="str">
+        <x:v>skills.indicator</x:v>
+      </x:c>
+      <x:c r="C2843" s="137" t="str">
+        <x:v>Интерфейс сайта</x:v>
+      </x:c>
+      <x:c r="D2843" s="138" t="str"/>
+      <x:c r="E2843" s="138" t="str">
+        <x:v>Legacy next-point indicator: </x:v>
+      </x:c>
+      <x:c r="F2843" s="138" t="str"/>
+      <x:c r="G2843" s="138" t="str"/>
+      <x:c r="H2843" s="139" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2307a5e74eb4215"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c0af64477a4a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): compact native inputs and panels with complete catalog regression coverage
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="186">
+  <cellXfs count="188">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -875,6 +875,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -883,8 +889,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2876" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I2876"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2883" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2883"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Раздел"/>
     <tableColumn id="2" name="ID (не менять)"/>
@@ -71940,6 +71946,153 @@
       </c>
       <c r="I2876" t="str" s="143"/>
     </row>
+    <row r="2877" ht="52" customHeight="1">
+      <c r="A2877" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2877" t="str" s="23">
+        <v>calculator.inputInvalid</v>
+      </c>
+      <c r="C2877" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2877" t="str" s="24"/>
+      <c r="E2877" s="186" t="str">
+        <v>Enter a whole number within this field’s limits. Esc cancels your edit.</v>
+      </c>
+      <c r="F2877" s="24" t="str"/>
+      <c r="G2877" s="24" t="str"/>
+      <c r="H2877" s="187" t="str">
+        <v>Введите целое число в пределах поля. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2877" s="143" t="str"/>
+    </row>
+    <row r="2878" ht="52" customHeight="1">
+      <c r="A2878" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2878" t="str" s="23">
+        <v>calculator.inputBudget</v>
+      </c>
+      <c r="C2878" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2878" t="str" s="24"/>
+      <c r="E2878" s="186" t="str">
+        <v>Not enough attribute points. The field shows the value the engine could allocate.</v>
+      </c>
+      <c r="F2878" s="24" t="str"/>
+      <c r="G2878" s="24" t="str"/>
+      <c r="H2878" s="187" t="str">
+        <v>Не хватает очков характеристик. В поле показано значение, на которое хватило очков.</v>
+      </c>
+      <c r="I2878" s="143" t="str"/>
+    </row>
+    <row r="2879" ht="52" customHeight="1">
+      <c r="A2879" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2879" t="str" s="23">
+        <v>calculator.levelInputHelp</v>
+      </c>
+      <c r="C2879" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2879" t="str" s="24"/>
+      <c r="E2879" s="186" t="str">
+        <v>Level 1–55. Press Enter or leave the field to apply; Esc cancels.</v>
+      </c>
+      <c r="F2879" s="24" t="str"/>
+      <c r="G2879" s="24" t="str"/>
+      <c r="H2879" s="187" t="str">
+        <v>Уровень 1–55. Enter или выход из поля применяет значение; Esc отменяет.</v>
+      </c>
+      <c r="I2879" s="143" t="str"/>
+    </row>
+    <row r="2880" ht="82" customHeight="1">
+      <c r="A2880" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2880" t="str" s="23">
+        <v>calculator.attributeInputHelp</v>
+      </c>
+      <c r="C2880" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2880" t="str" s="24"/>
+      <c r="E2880" s="186" t="str">
+        <v>Base attribute before equipment bonuses. Race minimum, maximum 99 and available points apply. Enter applies; Esc cancels.</v>
+      </c>
+      <c r="F2880" s="24" t="str"/>
+      <c r="G2880" s="24" t="str"/>
+      <c r="H2880" s="187" t="str">
+        <v>Базовая характеристика без бонусов экипировки. Минимум зависит от расы, максимум 99; нужны свободные очки. Enter применяет, Esc отменяет.</v>
+      </c>
+      <c r="I2880" s="143" t="str"/>
+    </row>
+    <row r="2881" ht="52" customHeight="1">
+      <c r="A2881" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2881" t="str" s="23">
+        <v>calculator.totalWithBonuses</v>
+      </c>
+      <c r="C2881" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2881" t="str" s="24"/>
+      <c r="E2881" s="186" t="str">
+        <v>Total including equipment and other bonuses</v>
+      </c>
+      <c r="F2881" s="24" t="str"/>
+      <c r="G2881" s="24" t="str"/>
+      <c r="H2881" s="187" t="str">
+        <v>Итог с бонусами экипировки и другими эффектами</v>
+      </c>
+      <c r="I2881" s="143" t="str"/>
+    </row>
+    <row r="2882" ht="52" customHeight="1">
+      <c r="A2882" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2882" t="str" s="23">
+        <v>compare.hideIdentical</v>
+      </c>
+      <c r="C2882" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2882" t="str" s="24"/>
+      <c r="E2882" s="186" t="str">
+        <v>Hide identical stats</v>
+      </c>
+      <c r="F2882" s="24" t="str"/>
+      <c r="G2882" s="24" t="str"/>
+      <c r="H2882" s="187" t="str">
+        <v>Скрыть одинаковые характеристики</v>
+      </c>
+      <c r="I2882" s="143" t="str"/>
+    </row>
+    <row r="2883" ht="52" customHeight="1">
+      <c r="A2883" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2883" t="str" s="23">
+        <v>compare.allIdentical</v>
+      </c>
+      <c r="C2883" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2883" t="str" s="24"/>
+      <c r="E2883" s="186" t="str">
+        <v>All displayed stats are identical.</v>
+      </c>
+      <c r="F2883" s="24" t="str"/>
+      <c r="G2883" s="24" t="str"/>
+      <c r="H2883" s="187" t="str">
+        <v>Все показанные характеристики одинаковы.</v>
+      </c>
+      <c r="I2883" s="143" t="str"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Modern 3.03: compact native controls and understandable admin editing (#30)
* docs: record accepted Modern 3.02 and next native learning investigation

* feat(admin): show live characteristics and validate private edit previews

* feat(ui): compact native inputs and panels with complete catalog regression coverage

* docs(ci): describe Modern 3.03 acceptance and beginner editing workflow

* fix(admin): keep publication actions clear of current-record content

* fix(admin): disclose unresolved source markers without fabricating bonuses

* fix(ui): reserve readable skill-name columns across desktop font fallbacks

* fix(ui): fit complete Horsemanship label without shrinking step targets

* fix(calculator): preserve edited Waist Belt bonuses and accurate text-line checks
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="186">
+  <cellXfs count="188">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -875,6 +875,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -883,8 +889,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2876" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I2876"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2883" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2883"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Раздел"/>
     <tableColumn id="2" name="ID (не менять)"/>
@@ -71940,6 +71946,153 @@
       </c>
       <c r="I2876" t="str" s="143"/>
     </row>
+    <row r="2877" ht="52" customHeight="1">
+      <c r="A2877" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2877" t="str" s="23">
+        <v>calculator.inputInvalid</v>
+      </c>
+      <c r="C2877" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2877" t="str" s="24"/>
+      <c r="E2877" s="186" t="str">
+        <v>Enter a whole number within this field’s limits. Esc cancels your edit.</v>
+      </c>
+      <c r="F2877" s="24" t="str"/>
+      <c r="G2877" s="24" t="str"/>
+      <c r="H2877" s="187" t="str">
+        <v>Введите целое число в пределах поля. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2877" s="143" t="str"/>
+    </row>
+    <row r="2878" ht="52" customHeight="1">
+      <c r="A2878" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2878" t="str" s="23">
+        <v>calculator.inputBudget</v>
+      </c>
+      <c r="C2878" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2878" t="str" s="24"/>
+      <c r="E2878" s="186" t="str">
+        <v>Not enough attribute points. The field shows the value the engine could allocate.</v>
+      </c>
+      <c r="F2878" s="24" t="str"/>
+      <c r="G2878" s="24" t="str"/>
+      <c r="H2878" s="187" t="str">
+        <v>Не хватает очков характеристик. В поле показано значение, на которое хватило очков.</v>
+      </c>
+      <c r="I2878" s="143" t="str"/>
+    </row>
+    <row r="2879" ht="52" customHeight="1">
+      <c r="A2879" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2879" t="str" s="23">
+        <v>calculator.levelInputHelp</v>
+      </c>
+      <c r="C2879" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2879" t="str" s="24"/>
+      <c r="E2879" s="186" t="str">
+        <v>Level 1–55. Press Enter or leave the field to apply; Esc cancels.</v>
+      </c>
+      <c r="F2879" s="24" t="str"/>
+      <c r="G2879" s="24" t="str"/>
+      <c r="H2879" s="187" t="str">
+        <v>Уровень 1–55. Enter или выход из поля применяет значение; Esc отменяет.</v>
+      </c>
+      <c r="I2879" s="143" t="str"/>
+    </row>
+    <row r="2880" ht="82" customHeight="1">
+      <c r="A2880" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2880" t="str" s="23">
+        <v>calculator.attributeInputHelp</v>
+      </c>
+      <c r="C2880" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2880" t="str" s="24"/>
+      <c r="E2880" s="186" t="str">
+        <v>Base attribute before equipment bonuses. Race minimum, maximum 99 and available points apply. Enter applies; Esc cancels.</v>
+      </c>
+      <c r="F2880" s="24" t="str"/>
+      <c r="G2880" s="24" t="str"/>
+      <c r="H2880" s="187" t="str">
+        <v>Базовая характеристика без бонусов экипировки. Минимум зависит от расы, максимум 99; нужны свободные очки. Enter применяет, Esc отменяет.</v>
+      </c>
+      <c r="I2880" s="143" t="str"/>
+    </row>
+    <row r="2881" ht="52" customHeight="1">
+      <c r="A2881" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2881" t="str" s="23">
+        <v>calculator.totalWithBonuses</v>
+      </c>
+      <c r="C2881" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2881" t="str" s="24"/>
+      <c r="E2881" s="186" t="str">
+        <v>Total including equipment and other bonuses</v>
+      </c>
+      <c r="F2881" s="24" t="str"/>
+      <c r="G2881" s="24" t="str"/>
+      <c r="H2881" s="187" t="str">
+        <v>Итог с бонусами экипировки и другими эффектами</v>
+      </c>
+      <c r="I2881" s="143" t="str"/>
+    </row>
+    <row r="2882" ht="52" customHeight="1">
+      <c r="A2882" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2882" t="str" s="23">
+        <v>compare.hideIdentical</v>
+      </c>
+      <c r="C2882" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2882" t="str" s="24"/>
+      <c r="E2882" s="186" t="str">
+        <v>Hide identical stats</v>
+      </c>
+      <c r="F2882" s="24" t="str"/>
+      <c r="G2882" s="24" t="str"/>
+      <c r="H2882" s="187" t="str">
+        <v>Скрыть одинаковые характеристики</v>
+      </c>
+      <c r="I2882" s="143" t="str"/>
+    </row>
+    <row r="2883" ht="52" customHeight="1">
+      <c r="A2883" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2883" t="str" s="23">
+        <v>compare.allIdentical</v>
+      </c>
+      <c r="C2883" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2883" t="str" s="24"/>
+      <c r="E2883" s="186" t="str">
+        <v>All displayed stats are identical.</v>
+      </c>
+      <c r="F2883" s="24" t="str"/>
+      <c r="G2883" s="24" t="str"/>
+      <c r="H2883" s="187" t="str">
+        <v>Все показанные характеристики одинаковы.</v>
+      </c>
+      <c r="I2883" s="143" t="str"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(ui): compose compact Hybrid C workbench without hiding native controls
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="190">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -881,6 +881,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -889,8 +895,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2883" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I2883"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2888" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2888"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Раздел"/>
     <tableColumn id="2" name="ID (не менять)"/>
@@ -72093,6 +72099,111 @@
       </c>
       <c r="I2883" s="143" t="str"/>
     </row>
+    <row r="2884" ht="52" customHeight="1">
+      <c r="A2884" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2884" t="str" s="23">
+        <v>workbench.character</v>
+      </c>
+      <c r="C2884" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2884" t="str" s="24"/>
+      <c r="E2884" s="188" t="str">
+        <v>Character</v>
+      </c>
+      <c r="F2884" s="24" t="str"/>
+      <c r="G2884" s="24" t="str"/>
+      <c r="H2884" s="189" t="str">
+        <v>Персонаж</v>
+      </c>
+      <c r="I2884" s="143" t="str"/>
+    </row>
+    <row r="2885" ht="52" customHeight="1">
+      <c r="A2885" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2885" t="str" s="23">
+        <v>workbench.skills</v>
+      </c>
+      <c r="C2885" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2885" t="str" s="24"/>
+      <c r="E2885" s="188" t="str">
+        <v>Skills</v>
+      </c>
+      <c r="F2885" s="24" t="str"/>
+      <c r="G2885" s="24" t="str"/>
+      <c r="H2885" s="189" t="str">
+        <v>Умения</v>
+      </c>
+      <c r="I2885" s="143" t="str"/>
+    </row>
+    <row r="2886" ht="52" customHeight="1">
+      <c r="A2886" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2886" t="str" s="23">
+        <v>workbench.effects</v>
+      </c>
+      <c r="C2886" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2886" t="str" s="24"/>
+      <c r="E2886" s="188" t="str">
+        <v>Effects</v>
+      </c>
+      <c r="F2886" s="24" t="str"/>
+      <c r="G2886" s="24" t="str"/>
+      <c r="H2886" s="189" t="str">
+        <v>Эффекты</v>
+      </c>
+      <c r="I2886" s="143" t="str"/>
+    </row>
+    <row r="2887" ht="52" customHeight="1">
+      <c r="A2887" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2887" t="str" s="23">
+        <v>workbench.baseStats</v>
+      </c>
+      <c r="C2887" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2887" t="str" s="24"/>
+      <c r="E2887" s="188" t="str">
+        <v>Base stats</v>
+      </c>
+      <c r="F2887" s="24" t="str"/>
+      <c r="G2887" s="24" t="str"/>
+      <c r="H2887" s="189" t="str">
+        <v>Базовые характеристики</v>
+      </c>
+      <c r="I2887" s="143" t="str"/>
+    </row>
+    <row r="2888" ht="52" customHeight="1">
+      <c r="A2888" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2888" t="str" s="23">
+        <v>workbench.results</v>
+      </c>
+      <c r="C2888" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2888" t="str" s="24"/>
+      <c r="E2888" s="188" t="str">
+        <v>Calculated stats</v>
+      </c>
+      <c r="F2888" s="24" t="str"/>
+      <c r="G2888" s="24" t="str"/>
+      <c r="H2888" s="189" t="str">
+        <v>Результаты расчёта</v>
+      </c>
+      <c r="I2888" s="143" t="str"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix(ui): restore compact popups and field-specific feedback with consistent rows
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="194">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -887,6 +887,18 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -895,8 +907,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2888" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I2888"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2894" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2894"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Раздел"/>
     <tableColumn id="2" name="ID (не менять)"/>
@@ -72204,6 +72216,132 @@
       </c>
       <c r="I2888" s="143" t="str"/>
     </row>
+    <row r="2889" ht="52" customHeight="1">
+      <c r="A2889" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2889" t="str" s="23">
+        <v>calculator.inputMaximum</v>
+      </c>
+      <c r="C2889" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2889" t="str" s="24"/>
+      <c r="E2889" s="190" t="str">
+        <v>{field}: maximum {max}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2889" s="24" t="str"/>
+      <c r="G2889" s="24" t="str"/>
+      <c r="H2889" s="191" t="str">
+        <v>Максимальное значение поля «{field}» — {max}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2889" s="143" t="str"/>
+    </row>
+    <row r="2890" ht="52" customHeight="1">
+      <c r="A2890" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2890" t="str" s="23">
+        <v>calculator.inputMinimum</v>
+      </c>
+      <c r="C2890" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2890" t="str" s="24"/>
+      <c r="E2890" s="190" t="str">
+        <v>{field}: minimum {min}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2890" s="24" t="str"/>
+      <c r="G2890" s="24" t="str"/>
+      <c r="H2890" s="191" t="str">
+        <v>Минимальное значение поля «{field}» — {min}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2890" s="143" t="str"/>
+    </row>
+    <row r="2891" ht="52" customHeight="1">
+      <c r="A2891" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2891" t="str" s="23">
+        <v>calculator.inputWholeNumber</v>
+      </c>
+      <c r="C2891" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2891" t="str" s="24"/>
+      <c r="E2891" s="190" t="str">
+        <v>{field}: enter a whole number from {min} to {max}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2891" s="24" t="str"/>
+      <c r="G2891" s="24" t="str"/>
+      <c r="H2891" s="191" t="str">
+        <v>Для поля «{field}» введите целое число от {min} до {max}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2891" s="143" t="str"/>
+    </row>
+    <row r="2892" ht="52" customHeight="1">
+      <c r="A2892" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2892" t="str" s="23">
+        <v>calculator.inputRequired</v>
+      </c>
+      <c r="C2892" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2892" t="str" s="24"/>
+      <c r="E2892" s="190" t="str">
+        <v>{field}: enter a value from {min} to {max}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2892" s="24" t="str"/>
+      <c r="G2892" s="24" t="str"/>
+      <c r="H2892" s="191" t="str">
+        <v>Заполните поле «{field}»: целое число от {min} до {max}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2892" s="143" t="str"/>
+    </row>
+    <row r="2893" ht="52" customHeight="1">
+      <c r="A2893" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2893" t="str" s="23">
+        <v>calculator.inputBudgetForField</v>
+      </c>
+      <c r="C2893" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2893" t="str" s="24"/>
+      <c r="E2893" s="190" t="str">
+        <v>{field}: not enough attribute points. Applied value: {value}.</v>
+      </c>
+      <c r="F2893" s="24" t="str"/>
+      <c r="G2893" s="24" t="str"/>
+      <c r="H2893" s="191" t="str">
+        <v>Для поля «{field}» не хватает очков характеристик. Применено значение: {value}.</v>
+      </c>
+      <c r="I2893" s="143" t="str"/>
+    </row>
+    <row r="2894" ht="52" customHeight="1">
+      <c r="A2894" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2894" t="str" s="23">
+        <v>skills.listDisabled</v>
+      </c>
+      <c r="C2894" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2894" t="str" s="24"/>
+      <c r="E2894" s="192" t="str">
+        <v>The skill list is switched off. Enable it to show available and learned skills.</v>
+      </c>
+      <c r="F2894" s="24" t="str"/>
+      <c r="G2894" s="24" t="str"/>
+      <c r="H2894" s="193" t="str">
+        <v>Список умений выключен. Включите его, чтобы увидеть доступные и изученные умения.</v>
+      </c>
+      <c r="I2894" s="143" t="str"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Modern 3.04: compact Hybrid C composition (#33)
* feat(ui): compose compact Hybrid C workbench without hiding native controls

* docs: record Hybrid C decisions and verify deployment identity

* fix(ui): restore compact popups and field-specific feedback with consistent rows

* fix(ui): prevent inherited nowrap from clipping localized popup and section text

* fix(ui): give floating panels opaque surfaces and keep complete point budgets readable
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="194">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -881,6 +881,24 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -889,8 +907,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2883" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I2883"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2894" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2894"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Раздел"/>
     <tableColumn id="2" name="ID (не менять)"/>
@@ -72093,6 +72111,237 @@
       </c>
       <c r="I2883" s="143" t="str"/>
     </row>
+    <row r="2884" ht="52" customHeight="1">
+      <c r="A2884" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2884" t="str" s="23">
+        <v>workbench.character</v>
+      </c>
+      <c r="C2884" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2884" t="str" s="24"/>
+      <c r="E2884" s="188" t="str">
+        <v>Character</v>
+      </c>
+      <c r="F2884" s="24" t="str"/>
+      <c r="G2884" s="24" t="str"/>
+      <c r="H2884" s="189" t="str">
+        <v>Персонаж</v>
+      </c>
+      <c r="I2884" s="143" t="str"/>
+    </row>
+    <row r="2885" ht="52" customHeight="1">
+      <c r="A2885" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2885" t="str" s="23">
+        <v>workbench.skills</v>
+      </c>
+      <c r="C2885" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2885" t="str" s="24"/>
+      <c r="E2885" s="188" t="str">
+        <v>Skills</v>
+      </c>
+      <c r="F2885" s="24" t="str"/>
+      <c r="G2885" s="24" t="str"/>
+      <c r="H2885" s="189" t="str">
+        <v>Умения</v>
+      </c>
+      <c r="I2885" s="143" t="str"/>
+    </row>
+    <row r="2886" ht="52" customHeight="1">
+      <c r="A2886" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2886" t="str" s="23">
+        <v>workbench.effects</v>
+      </c>
+      <c r="C2886" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2886" t="str" s="24"/>
+      <c r="E2886" s="188" t="str">
+        <v>Effects</v>
+      </c>
+      <c r="F2886" s="24" t="str"/>
+      <c r="G2886" s="24" t="str"/>
+      <c r="H2886" s="189" t="str">
+        <v>Эффекты</v>
+      </c>
+      <c r="I2886" s="143" t="str"/>
+    </row>
+    <row r="2887" ht="52" customHeight="1">
+      <c r="A2887" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2887" t="str" s="23">
+        <v>workbench.baseStats</v>
+      </c>
+      <c r="C2887" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2887" t="str" s="24"/>
+      <c r="E2887" s="188" t="str">
+        <v>Base stats</v>
+      </c>
+      <c r="F2887" s="24" t="str"/>
+      <c r="G2887" s="24" t="str"/>
+      <c r="H2887" s="189" t="str">
+        <v>Базовые характеристики</v>
+      </c>
+      <c r="I2887" s="143" t="str"/>
+    </row>
+    <row r="2888" ht="52" customHeight="1">
+      <c r="A2888" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2888" t="str" s="23">
+        <v>workbench.results</v>
+      </c>
+      <c r="C2888" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2888" t="str" s="24"/>
+      <c r="E2888" s="188" t="str">
+        <v>Calculated stats</v>
+      </c>
+      <c r="F2888" s="24" t="str"/>
+      <c r="G2888" s="24" t="str"/>
+      <c r="H2888" s="189" t="str">
+        <v>Результаты расчёта</v>
+      </c>
+      <c r="I2888" s="143" t="str"/>
+    </row>
+    <row r="2889" ht="52" customHeight="1">
+      <c r="A2889" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2889" t="str" s="23">
+        <v>calculator.inputMaximum</v>
+      </c>
+      <c r="C2889" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2889" t="str" s="24"/>
+      <c r="E2889" s="190" t="str">
+        <v>{field}: maximum {max}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2889" s="24" t="str"/>
+      <c r="G2889" s="24" t="str"/>
+      <c r="H2889" s="191" t="str">
+        <v>Максимальное значение поля «{field}» — {max}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2889" s="143" t="str"/>
+    </row>
+    <row r="2890" ht="52" customHeight="1">
+      <c r="A2890" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2890" t="str" s="23">
+        <v>calculator.inputMinimum</v>
+      </c>
+      <c r="C2890" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2890" t="str" s="24"/>
+      <c r="E2890" s="190" t="str">
+        <v>{field}: minimum {min}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2890" s="24" t="str"/>
+      <c r="G2890" s="24" t="str"/>
+      <c r="H2890" s="191" t="str">
+        <v>Минимальное значение поля «{field}» — {min}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2890" s="143" t="str"/>
+    </row>
+    <row r="2891" ht="52" customHeight="1">
+      <c r="A2891" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2891" t="str" s="23">
+        <v>calculator.inputWholeNumber</v>
+      </c>
+      <c r="C2891" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2891" t="str" s="24"/>
+      <c r="E2891" s="190" t="str">
+        <v>{field}: enter a whole number from {min} to {max}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2891" s="24" t="str"/>
+      <c r="G2891" s="24" t="str"/>
+      <c r="H2891" s="191" t="str">
+        <v>Для поля «{field}» введите целое число от {min} до {max}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2891" s="143" t="str"/>
+    </row>
+    <row r="2892" ht="52" customHeight="1">
+      <c r="A2892" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2892" t="str" s="23">
+        <v>calculator.inputRequired</v>
+      </c>
+      <c r="C2892" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2892" t="str" s="24"/>
+      <c r="E2892" s="190" t="str">
+        <v>{field}: enter a value from {min} to {max}. Esc cancels your edit.</v>
+      </c>
+      <c r="F2892" s="24" t="str"/>
+      <c r="G2892" s="24" t="str"/>
+      <c r="H2892" s="191" t="str">
+        <v>Заполните поле «{field}»: целое число от {min} до {max}. Esc отменяет ввод.</v>
+      </c>
+      <c r="I2892" s="143" t="str"/>
+    </row>
+    <row r="2893" ht="52" customHeight="1">
+      <c r="A2893" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2893" t="str" s="23">
+        <v>calculator.inputBudgetForField</v>
+      </c>
+      <c r="C2893" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2893" t="str" s="24"/>
+      <c r="E2893" s="190" t="str">
+        <v>{field}: not enough attribute points. Applied value: {value}.</v>
+      </c>
+      <c r="F2893" s="24" t="str"/>
+      <c r="G2893" s="24" t="str"/>
+      <c r="H2893" s="191" t="str">
+        <v>Для поля «{field}» не хватает очков характеристик. Применено значение: {value}.</v>
+      </c>
+      <c r="I2893" s="143" t="str"/>
+    </row>
+    <row r="2894" ht="52" customHeight="1">
+      <c r="A2894" t="str" s="23">
+        <v>Интерфейс</v>
+      </c>
+      <c r="B2894" t="str" s="23">
+        <v>skills.listDisabled</v>
+      </c>
+      <c r="C2894" t="str" s="23">
+        <v>Интерфейс сайта</v>
+      </c>
+      <c r="D2894" t="str" s="24"/>
+      <c r="E2894" s="192" t="str">
+        <v>The skill list is switched off. Enable it to show available and learned skills.</v>
+      </c>
+      <c r="F2894" s="24" t="str"/>
+      <c r="G2894" s="24" t="str"/>
+      <c r="H2894" s="193" t="str">
+        <v>Список умений выключен. Включите его, чтобы увидеть доступные и изученные умения.</v>
+      </c>
+      <c r="I2894" s="143" t="str"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
i18n: add Russian calculator labels and hints
</commit_message>
<xml_diff>
--- a/localization/translations.xlsx
+++ b/localization/translations.xlsx
@@ -913,8 +913,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2904" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I2904"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TranslationsTable" displayName="TranslationsTable" ref="A1:I2908" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2908"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Раздел"/>
     <tableColumn id="2" name="ID (не менять)"/>
@@ -40334,7 +40334,11 @@
       <c r="G1557" s="24" t="str">
         <v>接近</v>
       </c>
-      <c r="H1557" s="25" t="str"/>
+      <c r="H1557" t="inlineStr" s="25">
+        <is>
+          <t>Ближний бой</t>
+        </is>
+      </c>
       <c r="I1557" s="143" t="str"/>
     </row>
     <row r="1558" ht="21" customHeight="1">
@@ -40359,7 +40363,11 @@
       <c r="G1558" s="24" t="str">
         <v>斬殺</v>
       </c>
-      <c r="H1558" s="25" t="str"/>
+      <c r="H1558" t="inlineStr" s="25">
+        <is>
+          <t>Секущий удар</t>
+        </is>
+      </c>
       <c r="I1558" s="143" t="str"/>
     </row>
     <row r="1559" ht="21" customHeight="1">
@@ -40384,7 +40392,11 @@
       <c r="G1559" s="24" t="str">
         <v>突刺</v>
       </c>
-      <c r="H1559" s="25" t="str"/>
+      <c r="H1559" t="inlineStr" s="25">
+        <is>
+          <t>Колющий удар</t>
+        </is>
+      </c>
       <c r="I1559" s="143" t="str"/>
     </row>
     <row r="1560" ht="21" customHeight="1">
@@ -40409,7 +40421,11 @@
       <c r="G1560" s="24" t="str">
         <v>揮砍</v>
       </c>
-      <c r="H1560" s="25" t="str"/>
+      <c r="H1560" t="inlineStr" s="25">
+        <is>
+          <t>Рубящий удар</t>
+        </is>
+      </c>
       <c r="I1560" s="143" t="str"/>
     </row>
     <row r="1561" ht="21" customHeight="1">
@@ -40434,7 +40450,11 @@
       <c r="G1561" s="24" t="str">
         <v>打擊</v>
       </c>
-      <c r="H1561" s="25" t="str"/>
+      <c r="H1561" t="inlineStr" s="25">
+        <is>
+          <t>Тяжелый удар</t>
+        </is>
+      </c>
       <c r="I1561" s="143" t="str"/>
     </row>
     <row r="1562" ht="21" customHeight="1">
@@ -40459,7 +40479,11 @@
       <c r="G1562" s="24" t="str">
         <v>防禦</v>
       </c>
-      <c r="H1562" s="25" t="str"/>
+      <c r="H1562" t="inlineStr" s="25">
+        <is>
+          <t>Оборона</t>
+        </is>
+      </c>
       <c r="I1562" s="143" t="str"/>
     </row>
     <row r="1563" ht="21" customHeight="1">
@@ -40484,7 +40508,11 @@
       <c r="G1563" s="24" t="str">
         <v>刺殺</v>
       </c>
-      <c r="H1563" s="25" t="str"/>
+      <c r="H1563" t="inlineStr" s="25">
+        <is>
+          <t>Тактика</t>
+        </is>
+      </c>
       <c r="I1563" s="143" t="str"/>
     </row>
     <row r="1564" ht="21" customHeight="1">
@@ -40509,7 +40537,11 @@
       <c r="G1564" s="24" t="str">
         <v>射擊</v>
       </c>
-      <c r="H1564" s="25" t="str"/>
+      <c r="H1564" t="inlineStr" s="25">
+        <is>
+          <t>Стрельба</t>
+        </is>
+      </c>
       <c r="I1564" s="143" t="str"/>
     </row>
     <row r="1565" ht="21" customHeight="1">
@@ -40534,7 +40566,11 @@
       <c r="G1565" s="24" t="str">
         <v>調合</v>
       </c>
-      <c r="H1565" s="25" t="str"/>
+      <c r="H1565" t="inlineStr" s="25">
+        <is>
+          <t>Ремесло</t>
+        </is>
+      </c>
       <c r="I1565" s="143" t="str"/>
     </row>
     <row r="1566" ht="21" customHeight="1">
@@ -40559,7 +40595,11 @@
       <c r="G1566" s="24" t="str">
         <v>暗殺</v>
       </c>
-      <c r="H1566" s="25" t="str"/>
+      <c r="H1566" t="inlineStr" s="25">
+        <is>
+          <t>Убийства</t>
+        </is>
+      </c>
       <c r="I1566" s="143" t="str"/>
     </row>
     <row r="1567" ht="21" customHeight="1">
@@ -40584,7 +40624,11 @@
       <c r="G1567" s="24" t="str">
         <v>機關</v>
       </c>
-      <c r="H1567" s="25" t="str"/>
+      <c r="H1567" t="inlineStr" s="25">
+        <is>
+          <t>Ловушки</t>
+        </is>
+      </c>
       <c r="I1567" s="143" t="str"/>
     </row>
     <row r="1568" ht="21" customHeight="1">
@@ -40609,7 +40653,11 @@
       <c r="G1568" s="24" t="str">
         <v>迴避</v>
       </c>
-      <c r="H1568" s="25" t="str"/>
+      <c r="H1568" t="inlineStr" s="25">
+        <is>
+          <t>Уклонение</t>
+        </is>
+      </c>
       <c r="I1568" s="143" t="str"/>
     </row>
     <row r="1569" ht="21" customHeight="1">
@@ -40634,7 +40682,11 @@
       <c r="G1569" s="24" t="str">
         <v>神聖</v>
       </c>
-      <c r="H1569" s="25" t="str"/>
+      <c r="H1569" t="inlineStr" s="25">
+        <is>
+          <t>Молитва</t>
+        </is>
+      </c>
       <c r="I1569" s="143" t="str"/>
     </row>
     <row r="1570" ht="21" customHeight="1">
@@ -40659,7 +40711,11 @@
       <c r="G1570" s="24" t="str">
         <v>慈愛</v>
       </c>
-      <c r="H1570" s="25" t="str"/>
+      <c r="H1570" t="inlineStr" s="25">
+        <is>
+          <t>Исцеление</t>
+        </is>
+      </c>
       <c r="I1570" s="143" t="str"/>
     </row>
     <row r="1571" ht="21" customHeight="1">
@@ -40684,7 +40740,11 @@
       <c r="G1571" s="24" t="str">
         <v>祝福</v>
       </c>
-      <c r="H1571" s="25" t="str"/>
+      <c r="H1571" t="inlineStr" s="25">
+        <is>
+          <t>Благословение</t>
+        </is>
+      </c>
       <c r="I1571" s="143" t="str"/>
     </row>
     <row r="1572" ht="21" customHeight="1">
@@ -40709,7 +40769,11 @@
       <c r="G1572" s="24" t="str">
         <v>退魔</v>
       </c>
-      <c r="H1572" s="25" t="str"/>
+      <c r="H1572" t="inlineStr" s="25">
+        <is>
+          <t>Экзорцизм</t>
+        </is>
+      </c>
       <c r="I1572" s="143" t="str"/>
     </row>
     <row r="1573" ht="21" customHeight="1">
@@ -40734,7 +40798,11 @@
       <c r="G1573" s="24" t="str">
         <v>聖歌</v>
       </c>
-      <c r="H1573" s="25" t="str"/>
+      <c r="H1573" t="inlineStr" s="25">
+        <is>
+          <t>Песнопения</t>
+        </is>
+      </c>
       <c r="I1573" s="143" t="str"/>
     </row>
     <row r="1574" ht="21" customHeight="1">
@@ -40759,7 +40827,11 @@
       <c r="G1574" s="24" t="str">
         <v>魔法</v>
       </c>
-      <c r="H1574" s="25" t="str"/>
+      <c r="H1574" t="inlineStr" s="25">
+        <is>
+          <t>Магия</t>
+        </is>
+      </c>
       <c r="I1574" s="143" t="str"/>
     </row>
     <row r="1575" ht="21" customHeight="1">
@@ -40784,7 +40856,11 @@
       <c r="G1575" s="24" t="str">
         <v>元素</v>
       </c>
-      <c r="H1575" s="25" t="str"/>
+      <c r="H1575" t="inlineStr" s="25">
+        <is>
+          <t>Магия стихий</t>
+        </is>
+      </c>
       <c r="I1575" s="143" t="str"/>
     </row>
     <row r="1576" ht="21" customHeight="1">
@@ -40809,7 +40885,11 @@
       <c r="G1576" s="24" t="str">
         <v>具現</v>
       </c>
-      <c r="H1576" s="25" t="str"/>
+      <c r="H1576" t="inlineStr" s="25">
+        <is>
+          <t>Воплощение</t>
+        </is>
+      </c>
       <c r="I1576" s="143" t="str"/>
     </row>
     <row r="1577" ht="21" customHeight="1">
@@ -40834,7 +40914,11 @@
       <c r="G1577" s="24" t="str">
         <v>暗黑</v>
       </c>
-      <c r="H1577" s="25" t="str"/>
+      <c r="H1577" t="inlineStr" s="25">
+        <is>
+          <t>Магия тьмы</t>
+        </is>
+      </c>
       <c r="I1577" s="143" t="str"/>
     </row>
     <row r="1578" ht="21" customHeight="1">
@@ -40859,7 +40943,11 @@
       <c r="G1578" s="24" t="str">
         <v>咒術</v>
       </c>
-      <c r="H1578" s="25" t="str"/>
+      <c r="H1578" t="inlineStr" s="25">
+        <is>
+          <t>Чары</t>
+        </is>
+      </c>
       <c r="I1578" s="143" t="str"/>
     </row>
     <row r="1579" ht="21" customHeight="1">
@@ -40884,7 +40972,11 @@
       <c r="G1579" s="24" t="str">
         <v>其他</v>
       </c>
-      <c r="H1579" s="25" t="str"/>
+      <c r="H1579" t="inlineStr" s="25">
+        <is>
+          <t>Особые</t>
+        </is>
+      </c>
       <c r="I1579" s="143" t="str"/>
     </row>
     <row r="1580" ht="21" customHeight="1">
@@ -40909,7 +41001,11 @@
       <c r="G1580" s="24" t="str">
         <v>種族</v>
       </c>
-      <c r="H1580" s="25" t="str"/>
+      <c r="H1580" t="inlineStr" s="25">
+        <is>
+          <t>Расовые</t>
+        </is>
+      </c>
       <c r="I1580" s="143" t="str"/>
     </row>
     <row r="1581" ht="21" customHeight="1">
@@ -40934,7 +41030,11 @@
       <c r="G1581" s="24" t="str">
         <v>騎乘</v>
       </c>
-      <c r="H1581" s="25" t="str"/>
+      <c r="H1581" t="inlineStr" s="25">
+        <is>
+          <t>Верховая езда</t>
+        </is>
+      </c>
       <c r="I1581" s="143" t="str"/>
     </row>
     <row r="1582" ht="21" customHeight="1">
@@ -52111,16 +52211,26 @@
       <c r="D2031" s="39" t="str">
         <v>Name.Text.Skill.Buff[5]</v>
       </c>
-      <c r="E2031" s="39" t="str">
-        <v>Enchantment (Magic attack)</v>
-      </c>
-      <c r="F2031" s="39" t="str">
-        <v>エンハンスエンチャント (魔法攻撃力)</v>
-      </c>
-      <c r="G2031" s="39" t="str">
-        <v>鋼力招來 (魔攻)</v>
-      </c>
-      <c r="H2031" s="40" t="str"/>
+      <c r="E2031" t="inlineStr" s="39">
+        <is>
+          <t>Enchant (MATK)</t>
+        </is>
+      </c>
+      <c r="F2031" t="inlineStr" s="39">
+        <is>
+          <t>エンハ (魔攻)</t>
+        </is>
+      </c>
+      <c r="G2031" t="inlineStr" s="39">
+        <is>
+          <t>鋼力招來 (魔攻)</t>
+        </is>
+      </c>
+      <c r="H2031" t="inlineStr" s="40">
+        <is>
+          <t>Усил МагАТК</t>
+        </is>
+      </c>
       <c r="I2031" s="143" t="str"/>
     </row>
     <row r="2032" ht="15" hidden="0" customHeight="1">
@@ -52136,16 +52246,26 @@
       <c r="D2032" s="39" t="str">
         <v>Name.Text.Skill.Buff[6]</v>
       </c>
-      <c r="E2032" s="39" t="str">
-        <v>Enchantment (Aura damage)</v>
-      </c>
-      <c r="F2032" s="39" t="str">
-        <v>エンハンスエンチャント (オーラダメージ)</v>
-      </c>
-      <c r="G2032" s="39" t="str">
-        <v>鋼力招來 (靈氣)</v>
-      </c>
-      <c r="H2032" s="40" t="str"/>
+      <c r="E2032" t="inlineStr" s="39">
+        <is>
+          <t>Enchant (Aura)</t>
+        </is>
+      </c>
+      <c r="F2032" t="inlineStr" s="39">
+        <is>
+          <t>エンハ (オーラ)</t>
+        </is>
+      </c>
+      <c r="G2032" t="inlineStr" s="39">
+        <is>
+          <t>鋼力招來 (靈氣)</t>
+        </is>
+      </c>
+      <c r="H2032" t="inlineStr" s="40">
+        <is>
+          <t>Усил Аура</t>
+        </is>
+      </c>
       <c r="I2032" s="143" t="str"/>
     </row>
     <row r="2033" ht="15" hidden="0" customHeight="1">
@@ -52161,16 +52281,26 @@
       <c r="D2033" s="39" t="str">
         <v>Name.Text.Skill.Buff[9]</v>
       </c>
-      <c r="E2033" s="39" t="str">
-        <v>Sage's Song (MATK)</v>
-      </c>
-      <c r="F2033" s="39" t="str">
-        <v>魔力の歌(魔攻)</v>
-      </c>
-      <c r="G2033" s="39" t="str">
-        <v>魔力之歌 (魔攻)</v>
-      </c>
-      <c r="H2033" s="40" t="str"/>
+      <c r="E2033" t="inlineStr" s="39">
+        <is>
+          <t>Sage's Son (MATK)</t>
+        </is>
+      </c>
+      <c r="F2033" t="inlineStr" s="39">
+        <is>
+          <t>魔力の歌(魔攻)</t>
+        </is>
+      </c>
+      <c r="G2033" t="inlineStr" s="39">
+        <is>
+          <t>魔力之歌 (魔攻)</t>
+        </is>
+      </c>
+      <c r="H2033" t="inlineStr" s="40">
+        <is>
+          <t>ПЕСН МагАТК</t>
+        </is>
+      </c>
       <c r="I2033" s="143" t="str"/>
     </row>
     <row r="2034" ht="15" hidden="0" customHeight="1">
@@ -52186,16 +52316,26 @@
       <c r="D2034" s="39" t="str">
         <v>Name.Text.Skill.Buff[10]</v>
       </c>
-      <c r="E2034" s="39" t="str">
-        <v>Sage's Song (Delay)</v>
-      </c>
-      <c r="F2034" s="39" t="str">
-        <v>魔力の歌(再使用)</v>
-      </c>
-      <c r="G2034" s="39" t="str">
-        <v>魔力之歌 (冷卻)</v>
-      </c>
-      <c r="H2034" s="40" t="str"/>
+      <c r="E2034" t="inlineStr" s="39">
+        <is>
+          <t>Sage's Son (Delay)</t>
+        </is>
+      </c>
+      <c r="F2034" t="inlineStr" s="39">
+        <is>
+          <t>魔力の歌(再使用)</t>
+        </is>
+      </c>
+      <c r="G2034" t="inlineStr" s="39">
+        <is>
+          <t>魔力之歌 (冷卻)</t>
+        </is>
+      </c>
+      <c r="H2034" t="inlineStr" s="40">
+        <is>
+          <t>ПЕСН Перезарядка</t>
+        </is>
+      </c>
       <c r="I2034" s="143" t="str"/>
     </row>
     <row r="2035" ht="15" hidden="0" customHeight="1">
@@ -52770,7 +52910,11 @@
       <c r="G2057" s="39" t="str">
         <v>HP</v>
       </c>
-      <c r="H2057" s="40" t="str"/>
+      <c r="H2057" t="inlineStr" s="40">
+        <is>
+          <t>ОЗ</t>
+        </is>
+      </c>
       <c r="I2057" s="143" t="str"/>
     </row>
     <row r="2058" ht="15" hidden="0" customHeight="1">
@@ -52795,7 +52939,11 @@
       <c r="G2058" s="39" t="str">
         <v>MP</v>
       </c>
-      <c r="H2058" s="40" t="str"/>
+      <c r="H2058" t="inlineStr" s="40">
+        <is>
+          <t>ОМ</t>
+        </is>
+      </c>
       <c r="I2058" s="143" t="str"/>
     </row>
     <row r="2059" ht="15" hidden="0" customHeight="1">
@@ -52820,7 +52968,11 @@
       <c r="G2059" s="39" t="str">
         <v>藥劑效果</v>
       </c>
-      <c r="H2059" s="40" t="str"/>
+      <c r="H2059" t="inlineStr" s="40">
+        <is>
+          <t>УВЕЛЗЕЛ</t>
+        </is>
+      </c>
       <c r="I2059" s="143" t="str"/>
     </row>
     <row r="2060" ht="15" hidden="0" customHeight="1">
@@ -52843,7 +52995,11 @@
         <v>ポーション回復量</v>
       </c>
       <c r="G2060" s="39" t="str"/>
-      <c r="H2060" s="40" t="str"/>
+      <c r="H2060" t="inlineStr" s="40">
+        <is>
+          <t>Восстанавливающее действие зелья</t>
+        </is>
+      </c>
       <c r="I2060" s="143" t="str"/>
     </row>
     <row r="2061" ht="15" hidden="0" customHeight="1">
@@ -52868,7 +53024,11 @@
       <c r="G2061" s="39" t="str">
         <v>HP技能</v>
       </c>
-      <c r="H2061" s="40" t="str"/>
+      <c r="H2061" t="inlineStr" s="40">
+        <is>
+          <t>% исцеления ОЗ</t>
+        </is>
+      </c>
       <c r="I2061" s="143" t="str"/>
     </row>
     <row r="2062" ht="15" hidden="0" customHeight="1">
@@ -52893,7 +53053,11 @@
       <c r="G2062" s="39" t="str">
         <v>HP恢復技能的效果</v>
       </c>
-      <c r="H2062" s="40" t="str"/>
+      <c r="H2062" t="inlineStr" s="40">
+        <is>
+          <t>% исцеленного ОЗ</t>
+        </is>
+      </c>
       <c r="I2062" s="143" t="str"/>
     </row>
     <row r="2063" ht="15" hidden="0" customHeight="1">
@@ -52918,7 +53082,11 @@
       <c r="G2063" s="39" t="str">
         <v>消耗MP</v>
       </c>
-      <c r="H2063" s="40" t="str"/>
+      <c r="H2063" t="inlineStr" s="40">
+        <is>
+          <t>Восст ОМ</t>
+        </is>
+      </c>
       <c r="I2063" s="143" t="str"/>
     </row>
     <row r="2064" ht="15" hidden="0" customHeight="1">
@@ -52939,7 +53107,11 @@
       </c>
       <c r="F2064" s="39" t="str"/>
       <c r="G2064" s="39" t="str"/>
-      <c r="H2064" s="40" t="str"/>
+      <c r="H2064" t="inlineStr" s="40">
+        <is>
+          <t>Восстановление ОМ</t>
+        </is>
+      </c>
       <c r="I2064" s="143" t="str"/>
     </row>
     <row r="2065" ht="15" hidden="0" customHeight="1">
@@ -52964,7 +53136,11 @@
       <c r="G2065" s="39" t="str">
         <v>攻/最大</v>
       </c>
-      <c r="H2065" s="40" t="str"/>
+      <c r="H2065" t="inlineStr" s="40">
+        <is>
+          <t>МаксАТК</t>
+        </is>
+      </c>
       <c r="I2065" s="143" t="str"/>
     </row>
     <row r="2066" ht="15" hidden="0" customHeight="1">
@@ -52989,7 +53165,11 @@
       <c r="G2066" s="39" t="str">
         <v>攻/前面</v>
       </c>
-      <c r="H2066" s="40" t="str"/>
+      <c r="H2066" t="inlineStr" s="40">
+        <is>
+          <t>Фронт+</t>
+        </is>
+      </c>
       <c r="I2066" s="143" t="str"/>
     </row>
     <row r="2067" ht="15" hidden="0" customHeight="1">
@@ -53014,7 +53194,11 @@
       <c r="G2067" s="39" t="str">
         <v>從正面進攻</v>
       </c>
-      <c r="H2067" s="40" t="str"/>
+      <c r="H2067" t="inlineStr" s="40">
+        <is>
+          <t>АТК / Фронтальная атака</t>
+        </is>
+      </c>
       <c r="I2067" s="143" t="str"/>
     </row>
     <row r="2068" ht="15" hidden="0" customHeight="1">
@@ -53039,7 +53223,11 @@
       <c r="G2068" s="39" t="str">
         <v>攻/後面</v>
       </c>
-      <c r="H2068" s="40" t="str"/>
+      <c r="H2068" t="inlineStr" s="40">
+        <is>
+          <t>Спин+</t>
+        </is>
+      </c>
       <c r="I2068" s="143" t="str"/>
     </row>
     <row r="2069" ht="15" hidden="0" customHeight="1">
@@ -53064,7 +53252,11 @@
       <c r="G2069" s="39" t="str">
         <v>從背後攻擊</v>
       </c>
-      <c r="H2069" s="40" t="str"/>
+      <c r="H2069" t="inlineStr" s="40">
+        <is>
+          <t>АТК / Атака в спину</t>
+        </is>
+      </c>
       <c r="I2069" s="143" t="str"/>
     </row>
     <row r="2070" ht="15" hidden="0" customHeight="1">
@@ -53089,7 +53281,11 @@
       <c r="G2070" s="39" t="str">
         <v>魔攻</v>
       </c>
-      <c r="H2070" s="40" t="str"/>
+      <c r="H2070" t="inlineStr" s="40">
+        <is>
+          <t>МагАТК</t>
+        </is>
+      </c>
       <c r="I2070" s="143" t="str"/>
     </row>
     <row r="2071" ht="15" hidden="0" customHeight="1">
@@ -53114,7 +53310,11 @@
       <c r="G2071" s="39" t="str">
         <v>魔法攻擊</v>
       </c>
-      <c r="H2071" s="40" t="str"/>
+      <c r="H2071" t="inlineStr" s="40">
+        <is>
+          <t>Магическая атака</t>
+        </is>
+      </c>
       <c r="I2071" s="143" t="str"/>
     </row>
     <row r="2072" ht="15" hidden="0" customHeight="1">
@@ -53139,7 +53339,11 @@
       <c r="G2072" s="39" t="str">
         <v>防禦</v>
       </c>
-      <c r="H2072" s="40" t="str"/>
+      <c r="H2072" t="inlineStr" s="40">
+        <is>
+          <t>ЗАЩИТА</t>
+        </is>
+      </c>
       <c r="I2072" s="143" t="str"/>
     </row>
     <row r="2073" ht="15" hidden="0" customHeight="1">
@@ -53164,7 +53368,11 @@
       <c r="G2073" s="39" t="str">
         <v>防/前面</v>
       </c>
-      <c r="H2073" s="40" t="str"/>
+      <c r="H2073" t="inlineStr" s="40">
+        <is>
+          <t>ФРОНТ Сопр</t>
+        </is>
+      </c>
       <c r="I2073" s="143" t="str"/>
     </row>
     <row r="2074" ht="15" hidden="0" customHeight="1">
@@ -53189,7 +53397,11 @@
       <c r="G2074" s="39" t="str">
         <v>從前面物理傷害</v>
       </c>
-      <c r="H2074" s="40" t="str"/>
+      <c r="H2074" t="inlineStr" s="40">
+        <is>
+          <t>Уменьшение получаемого урона от фронтальных атак</t>
+        </is>
+      </c>
       <c r="I2074" s="143" t="str"/>
     </row>
     <row r="2075" ht="15" hidden="0" customHeight="1">
@@ -53214,7 +53426,11 @@
       <c r="G2075" s="39" t="str">
         <v>防/後面</v>
       </c>
-      <c r="H2075" s="40" t="str"/>
+      <c r="H2075" t="inlineStr" s="40">
+        <is>
+          <t>СПИН Сопр</t>
+        </is>
+      </c>
       <c r="I2075" s="143" t="str"/>
     </row>
     <row r="2076" ht="15" hidden="0" customHeight="1">
@@ -53239,7 +53455,11 @@
       <c r="G2076" s="39" t="str">
         <v>從後面物理傷害</v>
       </c>
-      <c r="H2076" s="40" t="str"/>
+      <c r="H2076" t="inlineStr" s="40">
+        <is>
+          <t>Уменьшение получаемого урона от атак в спину</t>
+        </is>
+      </c>
       <c r="I2076" s="143" t="str"/>
     </row>
     <row r="2077" ht="15" hidden="0" customHeight="1">
@@ -53264,7 +53484,11 @@
       <c r="G2077" s="39" t="str">
         <v>物理傷害</v>
       </c>
-      <c r="H2077" s="40" t="str"/>
+      <c r="H2077" t="inlineStr" s="40">
+        <is>
+          <t>Физ СОПР</t>
+        </is>
+      </c>
       <c r="I2077" s="143" t="str"/>
     </row>
     <row r="2078" ht="15" hidden="0" customHeight="1">
@@ -53287,7 +53511,11 @@
         <v>被物理ダメージ</v>
       </c>
       <c r="G2078" s="39" t="str"/>
-      <c r="H2078" s="40" t="str"/>
+      <c r="H2078" t="inlineStr" s="40">
+        <is>
+          <t>Снижение получаемого физического урона</t>
+        </is>
+      </c>
       <c r="I2078" s="143" t="str"/>
     </row>
     <row r="2079" ht="15" hidden="0" customHeight="1">
@@ -53312,7 +53540,11 @@
       <c r="G2079" s="39" t="str">
         <v>物理傷害</v>
       </c>
-      <c r="H2079" s="40" t="str"/>
+      <c r="H2079" t="inlineStr" s="40">
+        <is>
+          <t>ФИЗ Сопр</t>
+        </is>
+      </c>
       <c r="I2079" s="143" t="str"/>
     </row>
     <row r="2080" ht="15" hidden="0" customHeight="1">
@@ -53335,7 +53567,11 @@
         <v>被物理ダメージ</v>
       </c>
       <c r="G2080" s="39" t="str"/>
-      <c r="H2080" s="40" t="str"/>
+      <c r="H2080" t="inlineStr" s="40">
+        <is>
+          <t>Уменьшение получаемого физического урона</t>
+        </is>
+      </c>
       <c r="I2080" s="143" t="str"/>
     </row>
     <row r="2081" ht="15" hidden="0" customHeight="1">
@@ -53360,7 +53596,11 @@
       <c r="G2081" s="39" t="str">
         <v>魔法傷害</v>
       </c>
-      <c r="H2081" s="40" t="str"/>
+      <c r="H2081" t="inlineStr" s="40">
+        <is>
+          <t>МАГ Сопр</t>
+        </is>
+      </c>
       <c r="I2081" s="143" t="str"/>
     </row>
     <row r="2082" ht="15" hidden="0" customHeight="1">
@@ -53383,7 +53623,11 @@
         <v>被魔法ダメージ</v>
       </c>
       <c r="G2082" s="39" t="str"/>
-      <c r="H2082" s="40" t="str"/>
+      <c r="H2082" t="inlineStr" s="40">
+        <is>
+          <t>Уменьшение получаемого магического урона</t>
+        </is>
+      </c>
       <c r="I2082" s="143" t="str"/>
     </row>
     <row r="2083" ht="15" hidden="0" customHeight="1">
@@ -53408,7 +53652,11 @@
       <c r="G2083" s="39" t="str">
         <v>命中</v>
       </c>
-      <c r="H2083" s="40" t="str"/>
+      <c r="H2083" t="inlineStr" s="40">
+        <is>
+          <t>Точность</t>
+        </is>
+      </c>
       <c r="I2083" s="143" t="str"/>
     </row>
     <row r="2084" ht="15" hidden="0" customHeight="1">
@@ -53433,7 +53681,11 @@
       <c r="G2084" s="39" t="str">
         <v>命/前面</v>
       </c>
-      <c r="H2084" s="40" t="str"/>
+      <c r="H2084" t="inlineStr" s="40">
+        <is>
+          <t>ТОЧН</t>
+        </is>
+      </c>
       <c r="I2084" s="143" t="str"/>
     </row>
     <row r="2085" ht="15" hidden="0" customHeight="1">
@@ -53458,7 +53710,11 @@
       <c r="G2085" s="39" t="str">
         <v>當從正面攻擊命中</v>
       </c>
-      <c r="H2085" s="40" t="str"/>
+      <c r="H2085" t="inlineStr" s="40">
+        <is>
+          <t>Точность</t>
+        </is>
+      </c>
       <c r="I2085" s="143" t="str"/>
     </row>
     <row r="2086" ht="15" hidden="0" customHeight="1">
@@ -53483,7 +53739,11 @@
       <c r="G2086" s="39" t="str">
         <v>暴擊率</v>
       </c>
-      <c r="H2086" s="40" t="str"/>
+      <c r="H2086" t="inlineStr" s="40">
+        <is>
+          <t>ШК</t>
+        </is>
+      </c>
       <c r="I2086" s="143" t="str"/>
     </row>
     <row r="2087" ht="15" hidden="0" customHeight="1">
@@ -53506,7 +53766,11 @@
         <v>クリティカル発生率</v>
       </c>
       <c r="G2087" s="39" t="str"/>
-      <c r="H2087" s="40" t="str"/>
+      <c r="H2087" t="inlineStr" s="40">
+        <is>
+          <t>Шанс критической атаки</t>
+        </is>
+      </c>
       <c r="I2087" s="143" t="str"/>
     </row>
     <row r="2088" ht="15" hidden="0" customHeight="1">
@@ -53531,7 +53795,11 @@
       <c r="G2088" s="39" t="str">
         <v>暴擊威力</v>
       </c>
-      <c r="H2088" s="40" t="str"/>
+      <c r="H2088" t="inlineStr" s="40">
+        <is>
+          <t>Крит УРОН</t>
+        </is>
+      </c>
       <c r="I2088" s="143" t="str"/>
     </row>
     <row r="2089" ht="15" hidden="0" customHeight="1">
@@ -53556,7 +53824,11 @@
       <c r="G2089" s="39" t="str">
         <v>暴擊威力</v>
       </c>
-      <c r="H2089" s="40" t="str"/>
+      <c r="H2089" t="inlineStr" s="40">
+        <is>
+          <t>Критический урон</t>
+        </is>
+      </c>
       <c r="I2089" s="143" t="str"/>
     </row>
     <row r="2090" ht="15" hidden="0" customHeight="1">
@@ -53581,7 +53853,11 @@
       <c r="G2090" s="39" t="str">
         <v>迴避</v>
       </c>
-      <c r="H2090" s="40" t="str"/>
+      <c r="H2090" t="inlineStr" s="40">
+        <is>
+          <t>Уклонение</t>
+        </is>
+      </c>
       <c r="I2090" s="143" t="str"/>
     </row>
     <row r="2091" ht="15" hidden="0" customHeight="1">
@@ -53606,7 +53882,11 @@
       <c r="G2091" s="39" t="str">
         <v>防/暴擊</v>
       </c>
-      <c r="H2091" s="40" t="str"/>
+      <c r="H2091" t="inlineStr" s="40">
+        <is>
+          <t>КРИТ Сопр</t>
+        </is>
+      </c>
       <c r="I2091" s="143" t="str"/>
     </row>
     <row r="2092" ht="15" hidden="0" customHeight="1">
@@ -53631,7 +53911,11 @@
       <c r="G2092" s="39" t="str">
         <v>防/暴擊率</v>
       </c>
-      <c r="H2092" s="40" t="str"/>
+      <c r="H2092" t="inlineStr" s="40">
+        <is>
+          <t>Шанс получить критический удар; 0 - стандарт</t>
+        </is>
+      </c>
       <c r="I2092" s="143" t="str"/>
     </row>
     <row r="2093" ht="15" hidden="0" customHeight="1">
@@ -53656,7 +53940,11 @@
       <c r="G2093" s="39" t="str">
         <v>防/暴威</v>
       </c>
-      <c r="H2093" s="40" t="str"/>
+      <c r="H2093" t="inlineStr" s="40">
+        <is>
+          <t>КУРОН СОПР</t>
+        </is>
+      </c>
       <c r="I2093" s="143" t="str"/>
     </row>
     <row r="2094" ht="15" hidden="0" customHeight="1">
@@ -53681,7 +53969,11 @@
       <c r="G2094" s="39" t="str">
         <v>防/暴擊威力</v>
       </c>
-      <c r="H2094" s="40" t="str"/>
+      <c r="H2094" t="inlineStr" s="40">
+        <is>
+          <t>Снижение получаемого критического урона</t>
+        </is>
+      </c>
       <c r="I2094" s="143" t="str"/>
     </row>
     <row r="2095" ht="15" hidden="0" customHeight="1">
@@ -53706,7 +53998,11 @@
       <c r="G2095" s="39" t="str">
         <v>迴/近戰</v>
       </c>
-      <c r="H2095" s="40" t="str"/>
+      <c r="H2095" t="inlineStr" s="40">
+        <is>
+          <t>Ближ УКЛОН</t>
+        </is>
+      </c>
       <c r="I2095" s="143" t="str"/>
     </row>
     <row r="2096" ht="15" hidden="0" customHeight="1">
@@ -53731,7 +54027,11 @@
       <c r="G2096" s="39" t="str">
         <v>近戰迴避</v>
       </c>
-      <c r="H2096" s="40" t="str"/>
+      <c r="H2096" t="inlineStr" s="40">
+        <is>
+          <t>Уклонение от атак ближнего боя</t>
+        </is>
+      </c>
       <c r="I2096" s="143" t="str"/>
     </row>
     <row r="2097" ht="15" hidden="0" customHeight="1">
@@ -53756,7 +54056,11 @@
       <c r="G2097" s="39" t="str">
         <v>迴/遠程</v>
       </c>
-      <c r="H2097" s="40" t="str"/>
+      <c r="H2097" t="inlineStr" s="40">
+        <is>
+          <t>Дальн АТК УКЛОН</t>
+        </is>
+      </c>
       <c r="I2097" s="143" t="str"/>
     </row>
     <row r="2098" ht="15" hidden="0" customHeight="1">
@@ -53781,7 +54085,11 @@
       <c r="G2098" s="39" t="str">
         <v>遠程迴避</v>
       </c>
-      <c r="H2098" s="40" t="str"/>
+      <c r="H2098" t="inlineStr" s="40">
+        <is>
+          <t>Шанс уклониться от атаки дальнего боя</t>
+        </is>
+      </c>
       <c r="I2098" s="143" t="str"/>
     </row>
     <row r="2099" ht="15" hidden="0" customHeight="1">
@@ -53806,7 +54114,11 @@
       <c r="G2099" s="39" t="str">
         <v>迴/魔法</v>
       </c>
-      <c r="H2099" s="40" t="str"/>
+      <c r="H2099" t="inlineStr" s="40">
+        <is>
+          <t>Маг УКЛОН</t>
+        </is>
+      </c>
       <c r="I2099" s="143" t="str"/>
     </row>
     <row r="2100" ht="15" hidden="0" customHeight="1">
@@ -53831,7 +54143,11 @@
       <c r="G2100" s="39" t="str">
         <v>魔法攻擊迴避</v>
       </c>
-      <c r="H2100" s="40" t="str"/>
+      <c r="H2100" t="inlineStr" s="40">
+        <is>
+          <t>Уклонение от магии</t>
+        </is>
+      </c>
       <c r="I2100" s="143" t="str"/>
     </row>
     <row r="2101" ht="15" hidden="0" customHeight="1">
@@ -53856,7 +54172,11 @@
       <c r="G2101" s="39" t="str">
         <v>範/近戰</v>
       </c>
-      <c r="H2101" s="40" t="str"/>
+      <c r="H2101" t="inlineStr" s="40">
+        <is>
+          <t>Дист ближ АТК</t>
+        </is>
+      </c>
       <c r="I2101" s="143" t="str"/>
     </row>
     <row r="2102" ht="15" hidden="0" customHeight="1">
@@ -53881,7 +54201,11 @@
       <c r="G2102" s="39" t="str">
         <v>近戰武器範圍</v>
       </c>
-      <c r="H2102" s="40" t="str"/>
+      <c r="H2102" t="inlineStr" s="40">
+        <is>
+          <t>Дальность атак ближнего боя</t>
+        </is>
+      </c>
       <c r="I2102" s="143" t="str"/>
     </row>
     <row r="2103" ht="15" hidden="0" customHeight="1">
@@ -53906,7 +54230,11 @@
       <c r="G2103" s="39" t="str">
         <v>範/遠程</v>
       </c>
-      <c r="H2103" s="40" t="str"/>
+      <c r="H2103" t="inlineStr" s="40">
+        <is>
+          <t>Дист дальн АТК</t>
+        </is>
+      </c>
       <c r="I2103" s="143" t="str"/>
     </row>
     <row r="2104" ht="15" hidden="0" customHeight="1">
@@ -53931,7 +54259,11 @@
       <c r="G2104" s="39" t="str">
         <v>遠程武器射程</v>
       </c>
-      <c r="H2104" s="40" t="str"/>
+      <c r="H2104" t="inlineStr" s="40">
+        <is>
+          <t>Дальность атак дальнего боя</t>
+        </is>
+      </c>
       <c r="I2104" s="143" t="str"/>
     </row>
     <row r="2105" ht="15" hidden="0" customHeight="1">
@@ -53956,7 +54288,11 @@
       <c r="G2105" s="39" t="str">
         <v>火抗性</v>
       </c>
-      <c r="H2105" s="40" t="str"/>
+      <c r="H2105" t="inlineStr" s="40">
+        <is>
+          <t>ОГН Сопр</t>
+        </is>
+      </c>
       <c r="I2105" s="143" t="str"/>
     </row>
     <row r="2106" ht="15" hidden="0" customHeight="1">
@@ -53977,7 +54313,11 @@
       </c>
       <c r="F2106" s="39" t="str"/>
       <c r="G2106" s="39" t="str"/>
-      <c r="H2106" s="40" t="str"/>
+      <c r="H2106" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость огню</t>
+        </is>
+      </c>
       <c r="I2106" s="143" t="str"/>
     </row>
     <row r="2107" ht="15" hidden="0" customHeight="1">
@@ -54002,7 +54342,11 @@
       <c r="G2107" s="39" t="str">
         <v>攻擊速度</v>
       </c>
-      <c r="H2107" s="40" t="str"/>
+      <c r="H2107" t="inlineStr" s="40">
+        <is>
+          <t>СКР АТК</t>
+        </is>
+      </c>
       <c r="I2107" s="143" t="str"/>
     </row>
     <row r="2108" ht="15" hidden="0" customHeight="1">
@@ -54023,7 +54367,11 @@
       </c>
       <c r="F2108" s="39" t="str"/>
       <c r="G2108" s="39" t="str"/>
-      <c r="H2108" s="40" t="str"/>
+      <c r="H2108" t="inlineStr" s="40">
+        <is>
+          <t>Скорость атаки</t>
+        </is>
+      </c>
       <c r="I2108" s="143" t="str"/>
     </row>
     <row r="2109" ht="15" hidden="0" customHeight="1">
@@ -54048,7 +54396,11 @@
       <c r="G2109" s="39" t="str">
         <v>冰抗性</v>
       </c>
-      <c r="H2109" s="40" t="str"/>
+      <c r="H2109" t="inlineStr" s="40">
+        <is>
+          <t>ЛЕД Сопр</t>
+        </is>
+      </c>
       <c r="I2109" s="143" t="str"/>
     </row>
     <row r="2110" ht="15" hidden="0" customHeight="1">
@@ -54069,7 +54421,11 @@
       </c>
       <c r="F2110" s="39" t="str"/>
       <c r="G2110" s="39" t="str"/>
-      <c r="H2110" s="40" t="str"/>
+      <c r="H2110" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость магии льда</t>
+        </is>
+      </c>
       <c r="I2110" s="143" t="str"/>
     </row>
     <row r="2111" ht="15" hidden="0" customHeight="1">
@@ -54094,7 +54450,11 @@
       <c r="G2111" s="39" t="str">
         <v>詠唱速度</v>
       </c>
-      <c r="H2111" s="40" t="str"/>
+      <c r="H2111" t="inlineStr" s="40">
+        <is>
+          <t>СКР Каста</t>
+        </is>
+      </c>
       <c r="I2111" s="143" t="str"/>
     </row>
     <row r="2112" ht="15" hidden="0" customHeight="1">
@@ -54115,7 +54475,11 @@
       </c>
       <c r="F2112" s="39" t="str"/>
       <c r="G2112" s="39" t="str"/>
-      <c r="H2112" s="40" t="str"/>
+      <c r="H2112" t="inlineStr" s="40">
+        <is>
+          <t>Скорость применения умений</t>
+        </is>
+      </c>
       <c r="I2112" s="143" t="str"/>
     </row>
     <row r="2113" ht="15" hidden="0" customHeight="1">
@@ -54140,7 +54504,11 @@
       <c r="G2113" s="39" t="str">
         <v>詠唱時間</v>
       </c>
-      <c r="H2113" s="40" t="str"/>
+      <c r="H2113" t="inlineStr" s="40">
+        <is>
+          <t>ВремяКаст</t>
+        </is>
+      </c>
       <c r="I2113" s="143" t="str"/>
     </row>
     <row r="2114" ht="15" hidden="0" customHeight="1">
@@ -54161,7 +54529,11 @@
       </c>
       <c r="F2114" s="39" t="str"/>
       <c r="G2114" s="39" t="str"/>
-      <c r="H2114" s="40" t="str"/>
+      <c r="H2114" t="inlineStr" s="40">
+        <is>
+          <t>Уменьшение времени применения умений</t>
+        </is>
+      </c>
       <c r="I2114" s="143" t="str"/>
     </row>
     <row r="2115" ht="15" hidden="0" customHeight="1">
@@ -54186,7 +54558,11 @@
       <c r="G2115" s="39" t="str">
         <v>雷抗性</v>
       </c>
-      <c r="H2115" s="40" t="str"/>
+      <c r="H2115" t="inlineStr" s="40">
+        <is>
+          <t>МОЛН Сопр</t>
+        </is>
+      </c>
       <c r="I2115" s="143" t="str"/>
     </row>
     <row r="2116" ht="15" hidden="0" customHeight="1">
@@ -54207,7 +54583,11 @@
       </c>
       <c r="F2116" s="39" t="str"/>
       <c r="G2116" s="39" t="str"/>
-      <c r="H2116" s="40" t="str"/>
+      <c r="H2116" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость магии молнии</t>
+        </is>
+      </c>
       <c r="I2116" s="143" t="str"/>
     </row>
     <row r="2117" ht="15" hidden="0" customHeight="1">
@@ -54232,7 +54612,11 @@
       <c r="G2117" s="39" t="str">
         <v>冷卻時間</v>
       </c>
-      <c r="H2117" s="40" t="str"/>
+      <c r="H2117" t="inlineStr" s="40">
+        <is>
+          <t>Перезарядка</t>
+        </is>
+      </c>
       <c r="I2117" s="143" t="str"/>
     </row>
     <row r="2118" ht="15" hidden="0" customHeight="1">
@@ -54257,7 +54641,11 @@
       <c r="G2118" s="39" t="str">
         <v>毒抗性</v>
       </c>
-      <c r="H2118" s="40" t="str"/>
+      <c r="H2118" t="inlineStr" s="40">
+        <is>
+          <t>ЯД Сопр</t>
+        </is>
+      </c>
       <c r="I2118" s="143" t="str"/>
     </row>
     <row r="2119" ht="15" hidden="0" customHeight="1">
@@ -54278,7 +54666,11 @@
       </c>
       <c r="F2119" s="39" t="str"/>
       <c r="G2119" s="39" t="str"/>
-      <c r="H2119" s="40" t="str"/>
+      <c r="H2119" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость магии яда</t>
+        </is>
+      </c>
       <c r="I2119" s="143" t="str"/>
     </row>
     <row r="2120" ht="15" hidden="0" customHeight="1">
@@ -54303,7 +54695,11 @@
       <c r="G2120" s="39" t="str">
         <v>行走速度</v>
       </c>
-      <c r="H2120" s="40" t="str"/>
+      <c r="H2120" t="inlineStr" s="40">
+        <is>
+          <t>СКР Движ</t>
+        </is>
+      </c>
       <c r="I2120" s="143" t="str"/>
     </row>
     <row r="2121" ht="15" hidden="0" customHeight="1">
@@ -54324,7 +54720,11 @@
       </c>
       <c r="F2121" s="39" t="str"/>
       <c r="G2121" s="39" t="str"/>
-      <c r="H2121" s="40" t="str"/>
+      <c r="H2121" t="inlineStr" s="40">
+        <is>
+          <t>Скорость передвижения</t>
+        </is>
+      </c>
       <c r="I2121" s="143" t="str"/>
     </row>
     <row r="2122" ht="15" hidden="0" customHeight="1">
@@ -54349,7 +54749,11 @@
       <c r="G2122" s="39" t="str">
         <v>市/行走</v>
       </c>
-      <c r="H2122" s="40" t="str"/>
+      <c r="H2122" t="inlineStr" s="40">
+        <is>
+          <t>ГородСКРП</t>
+        </is>
+      </c>
       <c r="I2122" s="143" t="str"/>
     </row>
     <row r="2123" ht="15" hidden="0" customHeight="1">
@@ -54374,7 +54778,11 @@
       <c r="G2123" s="39" t="str">
         <v>速度變化的城市</v>
       </c>
-      <c r="H2123" s="40" t="str"/>
+      <c r="H2123" t="inlineStr" s="40">
+        <is>
+          <t>Скорость передвижения по городу</t>
+        </is>
+      </c>
       <c r="I2123" s="143" t="str"/>
     </row>
     <row r="2124" ht="15" hidden="0" customHeight="1">
@@ -54399,7 +54807,11 @@
       <c r="G2124" s="39" t="str">
         <v>魅惑抗性</v>
       </c>
-      <c r="H2124" s="40" t="str"/>
+      <c r="H2124" t="inlineStr" s="40">
+        <is>
+          <t>ЧАР Сопр</t>
+        </is>
+      </c>
       <c r="I2124" s="143" t="str"/>
     </row>
     <row r="2125" ht="15" hidden="0" customHeight="1">
@@ -54420,7 +54832,11 @@
       </c>
       <c r="F2125" s="39" t="str"/>
       <c r="G2125" s="39" t="str"/>
-      <c r="H2125" s="40" t="str"/>
+      <c r="H2125" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость магии чар</t>
+        </is>
+      </c>
       <c r="I2125" s="143" t="str"/>
     </row>
     <row r="2126" ht="15" hidden="0" customHeight="1">
@@ -54445,7 +54861,11 @@
       <c r="G2126" s="39" t="str">
         <v>光抗性</v>
       </c>
-      <c r="H2126" s="40" t="str"/>
+      <c r="H2126" t="inlineStr" s="40">
+        <is>
+          <t>СВЕТ Сопр</t>
+        </is>
+      </c>
       <c r="I2126" s="143" t="str"/>
     </row>
     <row r="2127" ht="15" hidden="0" customHeight="1">
@@ -54466,7 +54886,11 @@
       </c>
       <c r="F2127" s="39" t="str"/>
       <c r="G2127" s="39" t="str"/>
-      <c r="H2127" s="40" t="str"/>
+      <c r="H2127" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость магии света</t>
+        </is>
+      </c>
       <c r="I2127" s="143" t="str"/>
     </row>
     <row r="2128" ht="15" hidden="0" customHeight="1">
@@ -54491,7 +54915,11 @@
       <c r="G2128" s="39" t="str">
         <v>黑暗抗性</v>
       </c>
-      <c r="H2128" s="40" t="str"/>
+      <c r="H2128" t="inlineStr" s="40">
+        <is>
+          <t>ТЬМ Сопр</t>
+        </is>
+      </c>
       <c r="I2128" s="143" t="str"/>
     </row>
     <row r="2129" ht="15" hidden="0" customHeight="1">
@@ -54512,7 +54940,11 @@
       </c>
       <c r="F2129" s="39" t="str"/>
       <c r="G2129" s="39" t="str"/>
-      <c r="H2129" s="40" t="str"/>
+      <c r="H2129" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость тьме</t>
+        </is>
+      </c>
       <c r="I2129" s="143" t="str"/>
     </row>
     <row r="2130" ht="15" hidden="0" customHeight="1">
@@ -54537,7 +54969,11 @@
       <c r="G2130" s="39" t="str">
         <v>體抗性</v>
       </c>
-      <c r="H2130" s="40" t="str"/>
+      <c r="H2130" t="inlineStr" s="40">
+        <is>
+          <t>АНМСОСТТЕЛ Сопр</t>
+        </is>
+      </c>
       <c r="I2130" s="143" t="str"/>
     </row>
     <row r="2131" ht="24" hidden="0" customHeight="1">
@@ -54562,7 +54998,11 @@
       <c r="G2131" s="39" t="str">
         <v>異常體抗性</v>
       </c>
-      <c r="H2131" s="40" t="str"/>
+      <c r="H2131" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость аномальных состояний тела</t>
+        </is>
+      </c>
       <c r="I2131" s="143" t="str"/>
     </row>
     <row r="2132" ht="15" hidden="0" customHeight="1">
@@ -54587,7 +55027,11 @@
       <c r="G2132" s="39" t="str">
         <v>精神抗性</v>
       </c>
-      <c r="H2132" s="40" t="str"/>
+      <c r="H2132" t="inlineStr" s="40">
+        <is>
+          <t>АНМСОСТДУХ Сопр</t>
+        </is>
+      </c>
       <c r="I2132" s="143" t="str"/>
     </row>
     <row r="2133" ht="24" hidden="0" customHeight="1">
@@ -54612,7 +55056,11 @@
       <c r="G2133" s="39" t="str">
         <v>精神錯亂抗性</v>
       </c>
-      <c r="H2133" s="40" t="str"/>
+      <c r="H2133" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость аномальных состояний духа</t>
+        </is>
+      </c>
       <c r="I2133" s="143" t="str"/>
     </row>
     <row r="2134" ht="15" hidden="0" customHeight="1">
@@ -54637,7 +55085,11 @@
       <c r="G2134" s="39" t="str">
         <v>秘法抗性</v>
       </c>
-      <c r="H2134" s="40" t="str"/>
+      <c r="H2134" t="inlineStr" s="40">
+        <is>
+          <t>МАГ Сопр</t>
+        </is>
+      </c>
       <c r="I2134" s="143" t="str"/>
     </row>
     <row r="2135" ht="15" hidden="0" customHeight="1">
@@ -54658,7 +55110,11 @@
       </c>
       <c r="F2135" s="39" t="str"/>
       <c r="G2135" s="39" t="str"/>
-      <c r="H2135" s="40" t="str"/>
+      <c r="H2135" t="inlineStr" s="40">
+        <is>
+          <t>Сопротивляемость магии</t>
+        </is>
+      </c>
       <c r="I2135" s="143" t="str"/>
     </row>
     <row r="2136" ht="15" hidden="0" customHeight="1">
@@ -55108,7 +55564,11 @@
       <c r="G2153" s="39" t="str">
         <v>體力</v>
       </c>
-      <c r="H2153" s="40" t="str"/>
+      <c r="H2153" t="inlineStr" s="40">
+        <is>
+          <t>ВЫН</t>
+        </is>
+      </c>
       <c r="I2153" s="143" t="str"/>
     </row>
     <row r="2154" ht="15" hidden="0" customHeight="1">
@@ -55133,7 +55593,11 @@
       <c r="G2154" s="39" t="str">
         <v>力量</v>
       </c>
-      <c r="H2154" s="40" t="str"/>
+      <c r="H2154" t="inlineStr" s="40">
+        <is>
+          <t>СИЛ</t>
+        </is>
+      </c>
       <c r="I2154" s="143" t="str"/>
     </row>
     <row r="2155" ht="15" hidden="0" customHeight="1">
@@ -55158,7 +55622,11 @@
       <c r="G2155" s="39" t="str">
         <v>敏捷</v>
       </c>
-      <c r="H2155" s="40" t="str"/>
+      <c r="H2155" t="inlineStr" s="40">
+        <is>
+          <t>ПРВ</t>
+        </is>
+      </c>
       <c r="I2155" s="143" t="str"/>
     </row>
     <row r="2156" ht="15" hidden="0" customHeight="1">
@@ -55183,7 +55651,11 @@
       <c r="G2156" s="39" t="str">
         <v>技巧</v>
       </c>
-      <c r="H2156" s="40" t="str"/>
+      <c r="H2156" t="inlineStr" s="40">
+        <is>
+          <t>ЛВК</t>
+        </is>
+      </c>
       <c r="I2156" s="143" t="str"/>
     </row>
     <row r="2157" ht="15" hidden="0" customHeight="1">
@@ -55208,7 +55680,11 @@
       <c r="G2157" s="39" t="str">
         <v>靈感</v>
       </c>
-      <c r="H2157" s="40" t="str"/>
+      <c r="H2157" t="inlineStr" s="40">
+        <is>
+          <t>СД</t>
+        </is>
+      </c>
       <c r="I2157" s="143" t="str"/>
     </row>
     <row r="2158" ht="15" hidden="0" customHeight="1">
@@ -55233,7 +55709,11 @@
       <c r="G2158" s="39" t="str">
         <v>智慧</v>
       </c>
-      <c r="H2158" s="40" t="str"/>
+      <c r="H2158" t="inlineStr" s="40">
+        <is>
+          <t>ИНТ</t>
+        </is>
+      </c>
       <c r="I2158" s="143" t="str"/>
     </row>
     <row r="2159" ht="15" hidden="0" customHeight="1">
@@ -75185,6 +75665,194 @@
         </is>
       </c>
       <c r="I2904" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="2905" ht="15" hidden="0" customHeight="1">
+      <c r="A2905" t="inlineStr" s="38">
+        <is>
+          <t>Игра</t>
+        </is>
+      </c>
+      <c r="B2905" t="inlineStr" s="38">
+        <is>
+          <t>calculator.qualified_buff.5.hint</t>
+        </is>
+      </c>
+      <c r="C2905" t="inlineStr" s="38">
+        <is>
+          <t>Подсказка калькулятора</t>
+        </is>
+      </c>
+      <c r="D2905" t="inlineStr" s="39">
+        <is>
+          <t>Name.Text.Skill.Buff[5] @title</t>
+        </is>
+      </c>
+      <c r="E2905" t="inlineStr" s="39">
+        <is>
+          <t>Enchantment (Magic attack)</t>
+        </is>
+      </c>
+      <c r="F2905" t="inlineStr" s="39">
+        <is>
+          <t>エンハンスエンチャント (魔法攻撃力)</t>
+        </is>
+      </c>
+      <c r="G2905" t="inlineStr" s="39">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2905" t="inlineStr" s="40">
+        <is>
+          <t>Усиление урона магией</t>
+        </is>
+      </c>
+      <c r="I2905" t="inlineStr" s="143">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="2906" ht="15" hidden="0" customHeight="1">
+      <c r="A2906" t="inlineStr" s="38">
+        <is>
+          <t>Игра</t>
+        </is>
+      </c>
+      <c r="B2906" t="inlineStr" s="38">
+        <is>
+          <t>calculator.qualified_buff.6.hint</t>
+        </is>
+      </c>
+      <c r="C2906" t="inlineStr" s="38">
+        <is>
+          <t>Подсказка калькулятора</t>
+        </is>
+      </c>
+      <c r="D2906" t="inlineStr" s="39">
+        <is>
+          <t>Name.Text.Skill.Buff[6] @title</t>
+        </is>
+      </c>
+      <c r="E2906" t="inlineStr" s="39">
+        <is>
+          <t>Enchantment (Aura damage)</t>
+        </is>
+      </c>
+      <c r="F2906" t="inlineStr" s="39">
+        <is>
+          <t>エンハンスエンチャント (オーラダメージ)</t>
+        </is>
+      </c>
+      <c r="G2906" t="inlineStr" s="39">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2906" t="inlineStr" s="40">
+        <is>
+          <t>Усиление урона аурой</t>
+        </is>
+      </c>
+      <c r="I2906" t="inlineStr" s="143">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="2907" ht="15" hidden="0" customHeight="1">
+      <c r="A2907" t="inlineStr" s="38">
+        <is>
+          <t>Игра</t>
+        </is>
+      </c>
+      <c r="B2907" t="inlineStr" s="38">
+        <is>
+          <t>calculator.qualified_buff.9.hint</t>
+        </is>
+      </c>
+      <c r="C2907" t="inlineStr" s="38">
+        <is>
+          <t>Подсказка калькулятора</t>
+        </is>
+      </c>
+      <c r="D2907" t="inlineStr" s="39">
+        <is>
+          <t>Name.Text.Skill.Buff[9] @title</t>
+        </is>
+      </c>
+      <c r="E2907" t="inlineStr" s="39">
+        <is>
+          <t>Sage's Song (MATK)</t>
+        </is>
+      </c>
+      <c r="F2907" t="inlineStr" s="39">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2907" t="inlineStr" s="39">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2907" t="inlineStr" s="40">
+        <is>
+          <t>Усиление урона магией</t>
+        </is>
+      </c>
+      <c r="I2907" t="inlineStr" s="143">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="2908" ht="15" hidden="0" customHeight="1">
+      <c r="A2908" t="inlineStr" s="38">
+        <is>
+          <t>Игра</t>
+        </is>
+      </c>
+      <c r="B2908" t="inlineStr" s="38">
+        <is>
+          <t>calculator.qualified_buff.10.hint</t>
+        </is>
+      </c>
+      <c r="C2908" t="inlineStr" s="38">
+        <is>
+          <t>Подсказка калькулятора</t>
+        </is>
+      </c>
+      <c r="D2908" t="inlineStr" s="39">
+        <is>
+          <t>Name.Text.Skill.Buff[10] @title</t>
+        </is>
+      </c>
+      <c r="E2908" t="inlineStr" s="39">
+        <is>
+          <t>Sage's Song (Delay)</t>
+        </is>
+      </c>
+      <c r="F2908" t="inlineStr" s="39">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2908" t="inlineStr" s="39">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2908" t="inlineStr" s="40">
+        <is>
+          <t>Ускорение перезарядки умений</t>
+        </is>
+      </c>
+      <c r="I2908" t="inlineStr" s="143">
         <is>
           <t/>
         </is>

</xml_diff>